<commit_message>
Remove WISeR references from Medicare rows; use Noridian Auth Tool result
WISeR does not apply to 64772. The Medicare PA columns now cite the Noridian
Auth Tool result (no auth required) instead of the WISeR guide.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiByUV3Zo1mhZNaeehe8GC
</commit_message>
<xml_diff>
--- a/Code Research/CPT_64772_Routing_2026.xlsx
+++ b/Code Research/CPT_64772_Routing_2026.xlsx
@@ -602,7 +602,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -641,7 +640,7 @@
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>5. Arizona WISeR does NOT reach 64772 (NCD 160.1 WISeR codes = 64605/64610 only).</t>
+          <t>5. Medicare Part B: the Noridian Auth Tool shows no prior authorization required for 64772.</t>
         </is>
       </c>
     </row>
@@ -652,7 +651,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -710,12 +708,12 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Case-by-case under NCD 160.1. Document to L38801 facet-RFA criteria (dual MBB &gt;=80%, frequency limits). Not in WISeR.</t>
+          <t>Case-by-case under NCD 160.1. Document to L38801 facet-RFA criteria (dual MBB &gt;=80%, frequency limits).</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
         <is>
-          <t>Noridian PA Lookup screenshot</t>
+          <t>Noridian Auth Tool screenshot (no auth required)</t>
         </is>
       </c>
       <c r="F14" s="17" t="inlineStr">
@@ -1322,7 +1320,6 @@
     <mergeCell ref="A43:F43"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A7:F7"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="A31:F31"/>
@@ -1333,6 +1330,7 @@
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7869,27 +7867,27 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Noridian JF Part B Prior Authorization Lookup Tool (WISeR codes are loaded) - save a dated screenshot to the patient file</t>
+          <t>Noridian Auth Tool - result for 64772: no prior authorization required. Save a dated screenshot to the patient file.</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>No standing Part B PA program covers 64772. WISeR Model Provider &amp; Supplier Operational Guide (Arizona is a WISeR state; Noridian JF)</t>
+          <t>None - Medicare Part B has no prior-authorization requirement for 64772 (confirmed with the Noridian Auth Tool)</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>WISeR Guide v7.0 - Appendix A Table A2; Appendix C Table C2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>v7.0, 24 Jul 2026 (model runs 1 Jan 2026 - 31 Dec 2031)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>NO - the NCD 160.1 WISeR code set is 64605 and 64610 only (trigeminal). Associated codes (C2): 61790, 64605, 64610, 70450, 76000, 77002, 00222, 01991.</t>
+          <t>n/a - no PA list applies</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
@@ -7922,8 +7920,7 @@
           <t>NCD 160.1 covers lesions produced by 'surgical cutting of the nerve (rhizolysis), chemical destruction of the nerve, or by creation of a radio-frequency lesion' for 'chronic or acute pain arising from conditions such as terminal cancer or lumbar degenerative arthritis'; payment 'may be made ... when used in selected cases (concurred in by the Medicare Administrative Contractor's medical staff)'. No criteria list, no frequency limit, no covered-dx table. 'NO auth required' = no pre-service gate; it does NOT mean the claim is safe - every 64772 claim is exposed to medical review.
 L38801 / A58403 (Noridian JF, Arizona contracts 03101/03102) do not list 64772, but they govern facet denervation and a reviewer can apply them by analogy - DOCUMENT TO THEM: two diagnostic MBBs each with &gt;=80% relief of index pain; &gt;=3 months pain; failed conservative care; second block &gt;=2 weeks after the first; CT or fluoroscopic guidance only; one spinal region and 1-2 levels per session; max 2 RF sessions per spinal region per rolling 12 months; repeat only after &gt;=50% relief for &gt;=6 months; if &gt;=2 years since the last RFA, repeat the diagnostic blocks. Sedation (L38801 / A58403): routine moderate sedation, MAC, deep sedation or general anaesthesia for facet denervation is NOT reasonable and necessary; moderate sedation only case by case with documented necessity. L38801 lists as NOT reasonable &amp; necessary: non-thermal denervation (chemical, &lt;80 C, laser, cryoablation), prolotherapy, intra-facet implants. CORRECTION (round 2): the LCD is NOT silent on the endoscopic technique - L38801 (Analysis of Evidence): "An alternative method of denervation using an endoscopic approach (i.e., endoscopic dorsal ramus rhizotomy) has also been proposed. There is insufficient evidence in the published medical literature to determine the safety and efficacy of these emerging alternative modalities or approaches compared to thermal radiofrequency denervation." Endoscopic MBT is therefore outside the LCD's covered indications (thermal RF only) and is exposed to a not-reasonable-and-necessary denial on review. A58403: non-thermal denervation is reported with 64999 and is non-covered. A58403 ICD-10 list: for DENERVATION use M47.812-M47.817, M47.892-M47.897 or M48.12-M48.17 only - M53.82-M53.87 are flagged for facet cyst procedures, not ablation.
 NCCI (PTP v323r0, eff. 1 Oct 2026): 64772 is column 1 over 64490-64495, 62320-62327, 64479-64484 and 64400-64505 nerve blocks with modifier indicator 0 (no bypass) - same-session blocks are not separately payable. No PTP edit with 64633-64636 or 64625.
-RVU indicators: mult proc 2 (100/50/50 reduction for additional units/procedures), bilateral 0 (no 150% - report each nerve as a unit, RT/LT), assistant surgeon 2 (payable), co-surgeon 1 (with documentation), team 0.
-WISeR: 64772 is NOT a WISeR code (see N).</t>
+RVU indicators: mult proc 2 (100/50/50 reduction for additional units/procedures), bilateral 0 (no 150% - report each nerve as a unit, RT/LT), assistant surgeon 2 (payable), co-surgeon 1 (with documentation), team 0.</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
@@ -7982,7 +7979,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>No PA program. WISeR does not apply: the WISeR Guide states Railroad Medicare and Medicare Advantage beneficiaries are not impacted.</t>
+          <t>None - no prior-authorization program for 64772</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -9581,7 +9578,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
   </sheetData>
   <autoFilter ref="A1:V2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9594,7 +9590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -9610,6 +9606,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -9701,34 +9698,34 @@
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>WISeR Model Provider &amp; Supplier Operational Guide</t>
+          <t>Practitioner PTP edits for 64772</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>v7.0</t>
+          <t>v323r0</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>24 Jul 2026</t>
+          <t>Eff. 1 Oct 2026</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>cms.gov/priorities/innovation/files/wiser-provider-supplier-guide.pdf</t>
+          <t>Code Research/.../Medicare</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Practitioner PTP edits for 64772</t>
+          <t>Practitioner MUE 64772</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>v323r0</t>
+          <t>MUE 6 / MAI 3</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
@@ -9738,134 +9735,134 @@
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Medicare</t>
+          <t>Code Research/.../Medicare/MUE 64772 CMS</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>Practitioner MUE 64772</t>
+          <t>National PFS RVU file / ASC Addendum AA extracts</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>MUE 6 / MAI 3</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Oct 2026</t>
+          <t>Jan 2026</t>
         </is>
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Medicare/MUE 64772 CMS</t>
+          <t>Code Research/.../Medicare</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>National PFS RVU file / ASC Addendum AA extracts</t>
+          <t>AHCCCS FFS Physician Fee Schedule</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>FFY26</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>Jan 2026</t>
+          <t>File eff. 07/01/2026 (64772 rate date 10/1/2025)</t>
         </is>
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Medicare</t>
+          <t>Code Research/.../FY26_Final_PhysicianFeeSchedule.xlsx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>AHCCCS FFS Physician Fee Schedule</t>
+          <t>AZ Blue PA Requirements Code Lists</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>FFY26</t>
+          <t>All tabs incl. hidden</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>File eff. 07/01/2026 (64772 rate date 10/1/2025)</t>
+          <t>Updated 09/01/2026</t>
         </is>
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../FY26_Final_PhysicianFeeSchedule.xlsx</t>
+          <t>Payer's Prior Authorizations Articles/az-blue-prior-auth-code-lists.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>AZ Blue PA Requirements Code Lists</t>
+          <t>AZ Blue and TPA Jointly Administered Plans</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>All tabs incl. hidden</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>Updated 09/01/2026</t>
+          <t>As of 07/2026</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>Payer's Prior Authorizations Articles/az-blue-prior-auth-code-lists.xlsx</t>
+          <t>Plan Guides / PA Articles</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>AZ Blue and TPA Jointly Administered Plans</t>
+          <t>AZ Blue eviCore Programs FAQ</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>01-2024</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>As of 07/2026</t>
+          <t>Jan 2024</t>
         </is>
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>Plan Guides / PA Articles</t>
+          <t>Code Research/.../BCBS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>AZ Blue eviCore Programs FAQ</t>
+          <t>AZ Blue Ablation of Peripheral Nerves to Treat Pain</t>
         </is>
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>01-2024</t>
+          <t>O983.11</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>Jan 2024</t>
+          <t>Eff. 06/03/2026</t>
         </is>
       </c>
       <c r="D14" s="17" t="inlineStr">
@@ -9877,56 +9874,56 @@
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>AZ Blue Ablation of Peripheral Nerves to Treat Pain</t>
+          <t>MCG A-0218 / A-0695 / R-0056 / R-0058 working summaries</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>O983.11</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>Eff. 06/03/2026</t>
+          <t>Accessed 09/22/2026</t>
         </is>
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../BCBS</t>
+          <t>Code Research/.../BCBS (paraphrased summaries)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>MCG A-0218 / A-0695 / R-0056 / R-0058 working summaries</t>
+          <t>OptumCare Network of AZ - BCBS PA requirements</t>
         </is>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>OHNC-1-25-00929_09032026</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>Accessed 09/22/2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026</t>
         </is>
       </c>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../BCBS (paraphrased summaries)</t>
+          <t>PA Articles / Code Research/.../Optum</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>OptumCare Network of AZ - BCBS PA requirements</t>
+          <t>OptumCare Network of AZ - UHC MA PA and referral requirements</t>
         </is>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00929_09032026</t>
+          <t>OHNC-1-25-00928_08262026</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
@@ -9943,34 +9940,34 @@
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>OptumCare Network of AZ - UHC MA PA and referral requirements</t>
+          <t>OptumCare Network of AZ Provider Administrative Guide (delegation page)</t>
         </is>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00910_06182026</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>PA Articles / Code Research/.../Optum</t>
+          <t>Plan Guides/AZ_Optum Optum delegation.pdf</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>OptumCare Network of AZ Provider Administrative Guide (delegation page)</t>
+          <t>UHC QRG - Optum Care Arizona</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00910_06182026</t>
+          <t>PCA-4-26-00582-M&amp;R-QRG_05132026</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
@@ -9980,36 +9977,36 @@
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>Plan Guides/AZ_Optum Optum delegation.pdf</t>
+          <t>Code Research/.../Optum</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>UHC QRG - Optum Care Arizona</t>
+          <t>SCAN MA PA requirements</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>PCA-4-26-00582-M&amp;R-QRG_05132026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Rev. 1 Aug 2026</t>
         </is>
       </c>
       <c r="D20" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Optum</t>
+          <t>PA Articles</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>SCAN MA PA requirements</t>
+          <t>SCAN BCG0100 / BCG0111 / CCP0207 / CRP0420</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
@@ -10019,73 +10016,73 @@
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>Rev. 1 Aug 2026</t>
+          <t>5/28/2026; 5/6/2026; 11/20/2025; 5/28/2026</t>
         </is>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>PA Articles</t>
+          <t>Code Research/.../Optum</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>SCAN BCG0100 / BCG0111 / CCP0207 / CRP0420</t>
+          <t>Humana MA &amp; D-SNP PA and Notification List</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>790807ALL0725-C GHHMXVMEN</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>5/28/2026; 5/6/2026; 11/20/2025; 5/28/2026</t>
+          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
         </is>
       </c>
       <c r="D22" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Optum</t>
+          <t>PA Articles</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>Humana MA &amp; D-SNP PA and Notification List</t>
+          <t>Humana Neuroablative Techniques for Chronic Pain (MA)</t>
         </is>
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>790807ALL0725-C GHHMXVMEN</t>
+          <t>HUM-1168-008</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
+          <t>Eff. 08/06/2026</t>
         </is>
       </c>
       <c r="D23" s="17" t="inlineStr">
         <is>
-          <t>PA Articles</t>
+          <t>Code Research/.../Humana</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>Humana Neuroablative Techniques for Chronic Pain (MA)</t>
+          <t>Humana Injections for Pain Conditions (MA)</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>HUM-1168-008</t>
+          <t>HUM-1137-010</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>Eff. 08/06/2026</t>
+          <t>Eff. 09/01/2026</t>
         </is>
       </c>
       <c r="D24" s="17" t="inlineStr">
@@ -10097,34 +10094,34 @@
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>Humana Injections for Pain Conditions (MA)</t>
+          <t>UHC MA / Peoples Health PA requirements</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>HUM-1137-010</t>
+          <t>PCA-4-26-00416-Clinical-QRG_03022026</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>Eff. 09/01/2026</t>
+          <t>Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Humana</t>
+          <t>PA Articles</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
         <is>
-          <t>UHC MA / Peoples Health PA requirements</t>
+          <t>UHC Commercial advance notification / PA</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>PCA-4-26-00416-Clinical-QRG_03022026</t>
+          <t>PCA-1-26-00657-Clinical-QRG_04232026</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
@@ -10141,12 +10138,12 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>UHC Commercial advance notification / PA</t>
+          <t>UHC Individual Exchange PA</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>PCA-1-26-00657-Clinical-QRG_04232026</t>
+          <t>PCA-5-26-00416-Clinical-QRG_03022026</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
@@ -10163,12 +10160,12 @@
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>UHC Individual Exchange PA</t>
+          <t>UHC Community Plan AZ - ACC / DD / ALTCS PA</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>PCA-5-26-00416-Clinical-QRG_03022026</t>
+          <t>PCA-5/2/1-24-03748</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
@@ -10185,12 +10182,12 @@
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>UHC Community Plan AZ - ACC / DD / ALTCS PA</t>
+          <t>Surest PA requirements</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>PCA-5/2/1-24-03748</t>
+          <t>PCA-1-24-01406</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
@@ -10207,17 +10204,17 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Surest PA requirements</t>
+          <t>UHC West commercial PA (California product - not applicable in AZ)</t>
         </is>
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>PCA-1-24-01406</t>
+          <t>PCA-5-24-01315</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Sep 2026</t>
+          <t>Eff. 1 Apr 2026</t>
         </is>
       </c>
       <c r="D30" s="17" t="inlineStr">
@@ -10229,39 +10226,39 @@
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>UHC West commercial PA (California product - not applicable in AZ)</t>
+          <t>UHC Ablative Treatment for Spinal Pain (Commercial/IE)</t>
         </is>
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>PCA-5-24-01315</t>
+          <t>2026T0107II</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Apr 2026</t>
+          <t>Eff. 1 Feb 2026</t>
         </is>
       </c>
       <c r="D31" s="17" t="inlineStr">
         <is>
-          <t>PA Articles</t>
+          <t>Code Research/.../UHC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>UHC Ablative Treatment for Spinal Pain (Commercial/IE)</t>
+          <t>UHC Ablative Treatment for Spinal Pain (Community Plan)</t>
         </is>
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>2026T0107II</t>
+          <t>CS001.T</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Feb 2026</t>
+          <t>Eff. 1 Mar 2026</t>
         </is>
       </c>
       <c r="D32" s="17" t="inlineStr">
@@ -10273,17 +10270,17 @@
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>UHC Ablative Treatment for Spinal Pain (Community Plan)</t>
+          <t>UHC Facet Joint and MBB Injections (Commercial/IE)</t>
         </is>
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>CS001.T</t>
+          <t>2026T0004WW</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Mar 2026</t>
+          <t>Eff. 10 Sep 2026</t>
         </is>
       </c>
       <c r="D33" s="17" t="inlineStr">
@@ -10295,17 +10292,17 @@
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>UHC Facet Joint and MBB Injections (Commercial/IE)</t>
+          <t>UHC Pain Management (MA)</t>
         </is>
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>2026T0004WW</t>
+          <t>MMP070.12</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>Eff. 10 Sep 2026</t>
+          <t>Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="D34" s="17" t="inlineStr">
@@ -10317,105 +10314,105 @@
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>UHC Pain Management (MA)</t>
+          <t>AZ UHC Dual Complete / Dual Complete One Provider Manual</t>
         </is>
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>MMP070.12</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Sep 2026</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../UHC</t>
+          <t>Plan Guides</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>AZ UHC Dual Complete / Dual Complete One Provider Manual</t>
+          <t>NPPES record - Timothy A. Luke, MD</t>
         </is>
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>NPI 1437125846</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Last updated 2020-01-20</t>
         </is>
       </c>
       <c r="D36" s="17" t="inlineStr">
         <is>
-          <t>Plan Guides</t>
+          <t>NPPES registry</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>NPPES record - Timothy A. Luke, MD</t>
+          <t>AMA CPT Knowledge Base - endoscopic rhizotomy Q&amp;As (64999 / 64772)</t>
         </is>
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>NPI 1437125846</t>
+          <t>Paywalled</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>Last updated 2020-01-20</t>
+          <t>Nov 2019</t>
         </is>
       </c>
       <c r="D37" s="17" t="inlineStr">
         <is>
-          <t>NPPES registry</t>
+          <t>findacode.com/newsletters/ama-cpt-kb/ (previews only)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>AMA CPT Knowledge Base - endoscopic rhizotomy Q&amp;As (64999 / 64772)</t>
+          <t>AHCCCS AMPM 320-B (experimental services)</t>
         </is>
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>Paywalled</t>
+          <t>320-B</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>Nov 2019</t>
+          <t>Eff. 10/01/2022</t>
         </is>
       </c>
       <c r="D38" s="17" t="inlineStr">
         <is>
-          <t>findacode.com/newsletters/ama-cpt-kb/ (previews only)</t>
+          <t>Code Research/Criteria and Coverage Policies - Articles</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>AHCCCS AMPM 320-B (experimental services)</t>
+          <t>AHCCCS AMPM Exhibit 300-1 (covered services, special circumstances)</t>
         </is>
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>320-B</t>
+          <t>Exhibit 300-1</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>Eff. 10/01/2022</t>
+          <t>Rev. 07/09/2026</t>
         </is>
       </c>
       <c r="D39" s="17" t="inlineStr">
@@ -10427,17 +10424,17 @@
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>AHCCCS AMPM Exhibit 300-1 (covered services, special circumstances)</t>
+          <t>AHCCCS AMPM 810 FFS Utilization Management</t>
         </is>
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>Exhibit 300-1</t>
+          <t>810</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>Rev. 07/09/2026</t>
+          <t>Eff. 06/17/2026</t>
         </is>
       </c>
       <c r="D40" s="17" t="inlineStr">
@@ -10449,17 +10446,17 @@
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>AHCCCS AMPM 810 FFS Utilization Management</t>
+          <t>AHCCCS AMPM 820 FFS Prior Authorization</t>
         </is>
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>810</t>
+          <t>820</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>Eff. 06/17/2026</t>
+          <t>Eff. 07/16/2026</t>
         </is>
       </c>
       <c r="D41" s="17" t="inlineStr">
@@ -10471,73 +10468,73 @@
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>AHCCCS AMPM 820 FFS Prior Authorization</t>
+          <t>LCD Facet Joint Interventions (retired version)</t>
         </is>
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>820</t>
+          <t>L38803</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>Eff. 07/16/2026</t>
+          <t>Rev. eff. 07/17/2025 (retired)</t>
         </is>
       </c>
       <c r="D42" s="17" t="inlineStr">
         <is>
-          <t>Code Research/Criteria and Coverage Policies - Articles</t>
+          <t>Code Research/.../Medicare - text identical to L38801</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>LCD Facet Joint Interventions (retired version)</t>
+          <t>Response to Comments: Facet Joint Interventions</t>
         </is>
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>L38803</t>
+          <t>A59795</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>Rev. eff. 07/17/2025 (retired)</t>
+          <t>Orig. eff. 07/07/2024</t>
         </is>
       </c>
       <c r="D43" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Medicare - text identical to L38801</t>
+          <t>Code Research/.../Medicare</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>Response to Comments: Facet Joint Interventions</t>
+          <t>2026 UHC Care Provider Administrative Guide (Commercial, Exchange, MA chapters; Others ch. 1; Individual Exchange ch. 4)</t>
         </is>
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>A59795</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>Orig. eff. 07/07/2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="D44" s="17" t="inlineStr">
         <is>
-          <t>Code Research/.../Medicare</t>
+          <t>Plan Guides</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>2026 UHC Care Provider Administrative Guide (Commercial, Exchange, MA chapters; Others ch. 1; Individual Exchange ch. 4)</t>
+          <t>UHC 2026 Individual Exchange plans - Quick reference guide</t>
         </is>
       </c>
       <c r="B45" s="17" t="inlineStr">
@@ -10559,29 +10556,29 @@
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>UHC 2026 Individual Exchange plans - Quick reference guide</t>
+          <t>UHC Community Plan AZ member handbook excerpt</t>
         </is>
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="C46" s="17" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
       <c r="D46" s="17" t="inlineStr">
         <is>
-          <t>Plan Guides</t>
+          <t>Plan Guides/AZ_Medicaid_Handbook.pdf</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>UHC Community Plan AZ member handbook excerpt</t>
+          <t>HumanaMA.pdf / HumanaMS.pdf (Maricopa 85023 plan lists)</t>
         </is>
       </c>
       <c r="B47" s="17" t="inlineStr">
@@ -10591,51 +10588,51 @@
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Network update 09/18/2026</t>
         </is>
       </c>
       <c r="D47" s="17" t="inlineStr">
         <is>
-          <t>Plan Guides/AZ_Medicaid_Handbook.pdf</t>
+          <t>Plan Guides</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>HumanaMA.pdf / HumanaMS.pdf (Maricopa 85023 plan lists)</t>
+          <t>Humana Commercial PA list (stale)</t>
         </is>
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>399806ALL0224-A GCHM8R6EN</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>Network update 09/18/2026</t>
+          <t>Eff. 07/01/2024, rev. 12/10/2024</t>
         </is>
       </c>
       <c r="D48" s="17" t="inlineStr">
         <is>
-          <t>Plan Guides</t>
+          <t>PA Articles</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
         <is>
-          <t>Humana Commercial PA list (stale)</t>
+          <t>UHC Complete PA requirements</t>
         </is>
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>399806ALL0224-A GCHM8R6EN</t>
+          <t>PCA-1-25-02057</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>Eff. 07/01/2024, rev. 12/10/2024</t>
+          <t>Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="D49" s="17" t="inlineStr">
@@ -10647,17 +10644,17 @@
     <row r="50">
       <c r="A50" s="17" t="inlineStr">
         <is>
-          <t>UHC Complete PA requirements</t>
+          <t>UHC MA PA requirements - prior edition</t>
         </is>
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>PCA-1-25-02057</t>
+          <t>PCA-4-26-00416</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Sep 2026</t>
+          <t>Eff. 1 Aug 2026</t>
         </is>
       </c>
       <c r="D50" s="17" t="inlineStr">
@@ -10669,17 +10666,17 @@
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
         <is>
-          <t>UHC MA PA requirements - prior edition</t>
+          <t>Optum Behavioral Health - AZ Exchange PA list (not relevant to 64772)</t>
         </is>
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>PCA-4-26-00416</t>
+          <t>BH00798-2-24-QRG_01012025</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Aug 2026</t>
+          <t>Eff. 1 Jan 2026</t>
         </is>
       </c>
       <c r="D51" s="17" t="inlineStr">
@@ -10691,17 +10688,17 @@
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
         <is>
-          <t>Optum Behavioral Health - AZ Exchange PA list (not relevant to 64772)</t>
+          <t>Non-Arizona lists read and set aside: Oxford (NY/NJ/CT), NHP (FL), Mid-Atlantic (MD/DC/VA), UHC Community Plan FL, SCAN VillageHealth (CA)</t>
         </is>
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>BH00798-2-24-QRG_01012025</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026</t>
+          <t>Aug-Sep 2026</t>
         </is>
       </c>
       <c r="D52" s="17" t="inlineStr">
@@ -10713,7 +10710,7 @@
     <row r="53">
       <c r="A53" s="17" t="inlineStr">
         <is>
-          <t>Non-Arizona lists read and set aside: Oxford (NY/NJ/CT), NHP (FL), Mid-Atlantic (MD/DC/VA), UHC Community Plan FL, SCAN VillageHealth (CA)</t>
+          <t>Claims history: ALL Claims 2026-S1 - Master + monthly files; Job_Responsibilities_Inventory; code and timely-filing references</t>
         </is>
       </c>
       <c r="B53" s="17" t="inlineStr">
@@ -10723,32 +10720,10 @@
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>Aug-Sep 2026</t>
+          <t>DOS 01/2026-06/2026</t>
         </is>
       </c>
       <c r="D53" s="17" t="inlineStr">
-        <is>
-          <t>PA Articles</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
-        <is>
-          <t>Claims history: ALL Claims 2026-S1 - Master + monthly files; Job_Responsibilities_Inventory; code and timely-filing references</t>
-        </is>
-      </c>
-      <c r="B54" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C54" s="17" t="inlineStr">
-        <is>
-          <t>DOS 01/2026-06/2026</t>
-        </is>
-      </c>
-      <c r="D54" s="17" t="inlineStr">
         <is>
           <t>Repository root / Specialty Claims 2026-S1</t>
         </is>
@@ -10765,7 +10740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D864"/>
+  <dimension ref="A1:D877"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -29577,6 +29552,257 @@
         </is>
       </c>
     </row>
+    <row r="866">
+      <c r="A866" s="15" t="inlineStr">
+        <is>
+          <t>Round 3 - WISeR references removed (user correction: WISeR does not apply to 64772; Noridian Auth Tool = no auth), 23 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="17" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="B867" s="17" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="C867" s="17" t="inlineStr">
+        <is>
+          <t>Noridian JF Part B Prior Authorization Lookup Tool (WISeR codes are loaded) - save a dated screenshot to the patient file</t>
+        </is>
+      </c>
+      <c r="D867" s="17" t="inlineStr">
+        <is>
+          <t>Noridian Auth Tool - result for 64772: no prior authorization required. Save a dated screenshot to the patient file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="17" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="B868" s="17" t="inlineStr">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="C868" s="17" t="inlineStr">
+        <is>
+          <t>No standing Part B PA program covers 64772. WISeR Model Provider &amp; Supplier Operational Guide (Arizona is a WISeR state; Noridian JF)</t>
+        </is>
+      </c>
+      <c r="D868" s="17" t="inlineStr">
+        <is>
+          <t>None - Medicare Part B has no prior-authorization requirement for 64772 (confirmed with the Noridian Auth Tool)</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="17" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="B869" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C869" s="17" t="inlineStr">
+        <is>
+          <t>WISeR Guide v7.0 - Appendix A Table A2; Appendix C Table C2</t>
+        </is>
+      </c>
+      <c r="D869" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="17" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="B870" s="17" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="C870" s="17" t="inlineStr">
+        <is>
+          <t>v7.0, 24 Jul 2026 (model runs 1 Jan 2026 - 31 Dec 2031)</t>
+        </is>
+      </c>
+      <c r="D870" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="17" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="B871" s="17" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="C871" s="17" t="inlineStr">
+        <is>
+          <t>NO - the NCD 160.1 WISeR code set is 64605 and 64610 only (trigeminal). Associated codes (C2): 61790, 64605, 64610, 70450, 76000, 77002, 00222, 01991.</t>
+        </is>
+      </c>
+      <c r="D871" s="17" t="inlineStr">
+        <is>
+          <t>n/a - no PA list applies</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="17" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="B872" s="17" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C872" s="17" t="inlineStr">
+        <is>
+          <t>NCD 160.1 covers lesions produced by 'surgical cutting of the nerve (rhizolysis), chemical destruction of the nerve, or by creation of a radio-frequency lesion' for 'chronic or acute pain arising from conditions such as terminal cancer or lumbar degenerative arthritis'; payment 'may be made ... when used in selected cases (concurred in by the Medicare Administrative Contractor's medical staff)'. No criteria list, no frequency limit, no covered-dx table. 'NO auth required' = no pre-service gate; it does NOT mean the claim is safe - every 64772 claim is exposed to medical review.
+L38801 / A58403</t>
+        </is>
+      </c>
+      <c r="D872" s="17" t="inlineStr">
+        <is>
+          <t>NCD 160.1 covers lesions produced by 'surgical cutting of the nerve (rhizolysis), chemical destruction of the nerve, or by creation of a radio-frequency lesion' for 'chronic or acute pain arising from conditions such as terminal cancer or lumbar degenerative arthritis'; payment 'may be made ... when used in selected cases (concurred in by the Medicare Administrative Contractor's medical staff)'. No criteria list, no frequency limit, no covered-dx table. 'NO auth required' = no pre-service gate; it does NOT mean the claim is safe - every 64772 claim is exposed to medical review.
+L38801 / A58403</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="17" t="inlineStr">
+        <is>
+          <t>Medicare</t>
+        </is>
+      </c>
+      <c r="B873" s="17" t="inlineStr">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="C873" s="17" t="inlineStr">
+        <is>
+          <t>No PA program. WISeR does not apply: the WISeR Guide states Railroad Medicare and Medicare Advantage beneficiaries are not impacted.</t>
+        </is>
+      </c>
+      <c r="D873" s="17" t="inlineStr">
+        <is>
+          <t>None - no prior-authorization program for 64772</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B874" s="17" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="C874" s="17" t="inlineStr">
+        <is>
+          <t>5. Arizona WISeR does NOT reach 64772 (NCD 160.1 WISeR codes = 64605/64610 only).</t>
+        </is>
+      </c>
+      <c r="D874" s="17" t="inlineStr">
+        <is>
+          <t>5. Medicare Part B: the Noridian Auth Tool shows no prior authorization required for 64772.</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B875" s="17" t="inlineStr">
+        <is>
+          <t>D14</t>
+        </is>
+      </c>
+      <c r="C875" s="17" t="inlineStr">
+        <is>
+          <t>Case-by-case under NCD 160.1. Document to L38801 facet-RFA criteria (dual MBB &gt;=80%, frequency limits). Not in WISeR.</t>
+        </is>
+      </c>
+      <c r="D875" s="17" t="inlineStr">
+        <is>
+          <t>Case-by-case under NCD 160.1. Document to L38801 facet-RFA criteria (dual MBB &gt;=80%, frequency limits).</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B876" s="17" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="C876" s="17" t="inlineStr">
+        <is>
+          <t>Noridian PA Lookup screenshot</t>
+        </is>
+      </c>
+      <c r="D876" s="17" t="inlineStr">
+        <is>
+          <t>Noridian Auth Tool screenshot (no auth required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="17" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+      <c r="B877" s="17" t="inlineStr">
+        <is>
+          <t>A7:D7</t>
+        </is>
+      </c>
+      <c r="C877" s="17" t="inlineStr">
+        <is>
+          <t>WISeR Model Provider &amp; Supplier Operational Guide</t>
+        </is>
+      </c>
+      <c r="D877" s="17" t="inlineStr">
+        <is>
+          <t>ROW REMOVED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Re-match prior authorization documents to the correct payer rows
- UHC Complete and Surest get their own rows with their own PA lists
- UHC Community Plan split into ACC, DD and ALTCS rows, each with its own
  list and exact document ID
- Optum-delegated rows show the Optum list for Optum-direct providers and
  the health plan's list for everyone else
- Humana Medigap rows no longer cite the Humana MA list

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiByUV3Zo1mhZNaeehe8GC
</commit_message>
<xml_diff>
--- a/Code Research/CPT_64772_Routing_2026.xlsx
+++ b/Code Research/CPT_64772_Routing_2026.xlsx
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BCBS'!$A$1:$V$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Optum'!$A$1:$V$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'UnitedHealthcare'!$A$1:$V$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'UnitedHealthcare'!$A$1:$V$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Medicare'!$A$1:$U$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Humana'!$A$1:$V$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'AHCCCS FFS'!$A$1:$V$2</definedName>
@@ -762,7 +762,7 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>AZ Blue MA list 09/01/2026; Optum BCBS list OHNC-1-25-00929</t>
+          <t>AZ Blue MA list 09/01/2026; Optum BCBS list OHNC-1-25-00929 only for Optum-direct providers</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>None (excluded from Humana PA list); Medicare decides</t>
+          <t>None - not subject to PA; Medicare decides</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928 (eff. 1 Jan 2026, upd. 1 Sep 2026)</t>
+          <t>OHNC-1-25-00928 if Optum-direct; otherwise UHC MA list PCA-4-26-00416</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>PCA-1-26-00657; PCA-5-26-00416; 2026T0107II</t>
+          <t>PCA-1-26-00657 (Commercial); PCA-5-26-00416 (Exchange); PCA-1-25-02057 (UHC Complete); PCA-1-24-01406 (Surest); 2026T0107II</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>PCA-x-24-03748; CS001.T; PCA-4-26-00416</t>
+          <t>ACC PCA-5-24-003748; DD PCA-2-24-03748; ALTCS PCA-1-24-03748; Dual Complete PCA-4-26-00416; CS001.T</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
@@ -2101,22 +2101,22 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00929_09032026</t>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>NO - not listed. Pain Management section lists 62350-62362, 64490-64495, 64628/64629, 64633-64636 - not 64772</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
@@ -2305,22 +2305,22 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00929_09032026</t>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>NO - not listed (facet family 64490-64495 / 64633-64636 is listed)</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -2413,22 +2413,22 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00929_09032026</t>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>NO - not listed (facet family 64490-64495 / 64633-64636 is listed)</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
@@ -3448,22 +3448,22 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
@@ -3560,22 +3560,22 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O3" s="5" t="inlineStr">
@@ -3672,22 +3672,22 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O4" s="5" t="inlineStr">
@@ -3784,22 +3784,22 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr">
@@ -3896,22 +3896,22 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O6" s="5" t="inlineStr">
@@ -4008,22 +4008,22 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O7" s="5" t="inlineStr">
@@ -4120,22 +4120,22 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr">
@@ -4232,22 +4232,22 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
@@ -4344,22 +4344,22 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -4456,22 +4456,22 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr">
@@ -4568,22 +4568,22 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -4680,22 +4680,22 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -4792,22 +4792,22 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00928_08262026</t>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -4904,22 +4904,22 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00929_09032026</t>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>NO - absent (facet family is listed)</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr">
@@ -5016,22 +5016,22 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>OHNC-1-25-00929_09032026</t>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t>NO - absent (facet family is listed)</t>
+          <t>NO - absent from both lists</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -6079,7 +6079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -6987,7 +6987,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Navigate, Charter, Compass, NexusACO R / RB / RP, Freedom Granite Advantage-Saver EPO, UHC Complete</t>
+          <t>Navigate, Charter, Compass, NexusACO R / RB / RP, Freedom Granite Advantage-Saver EPO</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>64772 is absent from all four. But related techniques are AFFIRMATIVELY unproven and not medically necessary: pulsed RFA, endoscopic RFA / endoscopic rhizotomy, cryoablation, cooled RFA, chemical ablation, laser ablation. 'Ablation for treating sacroiliac pain is unproven and not medically necessary' - so 64625 is not covered commercially. Facet diagnostic block covered only when: facet loading pain on exam; no significant improvement (pain still &gt;=3/10) after &gt;=4 weeks conservative care; imaging excludes other causes; segment not fused; AND an RFA is being considered. Absence from a policy is NOT coverage. REFERRAL: gated plans need an ELECTRONIC PCP referral before the specialist visit (2026 UHC Administrative Guide, commercial chapter). UHC Complete has its own PA list (PCA-1-25-02057, eff. 1 Sep 2026): 64772 absent, but ALL unlisted codes incl. 64999 need PA and there is no non-emergent out-of-network coverage. Commercial "positive block" = &gt;=50% relief (2026T0004WW), not 80%.</t>
+          <t>64772 is absent from all four. But related techniques are AFFIRMATIVELY unproven and not medically necessary: pulsed RFA, endoscopic RFA / endoscopic rhizotomy, cryoablation, cooled RFA, chemical ablation, laser ablation. 'Ablation for treating sacroiliac pain is unproven and not medically necessary' - so 64625 is not covered commercially. Facet diagnostic block covered only when: facet loading pain on exam; no significant improvement (pain still &gt;=3/10) after &gt;=4 weeks conservative care; imaging excludes other causes; segment not fused; AND an RFA is being considered. Absence from a policy is NOT coverage. REFERRAL: gated plans need an ELECTRONIC PCP referral before the specialist visit (2026 UHC Administrative Guide, commercial chapter). UHC Complete now has its own row (own PA list). Commercial "positive block" = &gt;=50% relief (2026T0004WW), not 80%.</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
@@ -7283,7 +7283,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>UHC Community Plan - ACC, ACC-CRS, DD, DD-CRS, KidsCare, ALTCS-EPD</t>
+          <t>UHC Community Plan - AHCCCS Complete Care (ACC, incl. CRS-designated members)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -7307,22 +7307,22 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>NO - not on lists</t>
+          <t>NO - not on list</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal</t>
+          <t>UHC Provider Portal PA&amp;N tool, or 800-445-1638</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>UHC Community Plan of AZ PA requirements - ACC, Developmental Disabilities, Long Term Care</t>
+          <t>Prior authorization requirements for AHCCCS Complete Care (ACC) Medicaid - UnitedHealthcare Community Plan of Arizona</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>PCA-5-24-03748 (ACC); PCA-2-24-03748 (DD); PCA-1-24-03748 (ALTCS)</t>
+          <t>PCA-5-24-003748-Clinical-QRG_05192023</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>NO - absent from all three. 64490/64493 require PA (pain injections)</t>
+          <t>NO - absent. 64490 and 64493 require PA (pain injections &amp; management)</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t>64772 'TRANSECTION OR AVULSION OF OTHER SPINAL NERVE, EXTRADURAL' at $578.79 non-facility AND facility (rate parity); lower tier $405.15. 64999 is 'BR - by report'. COVERAGE CAVEAT, verbatim: 'the appearance on this website of a code and rate is not an indication of coverage, nor a guarantee of payment.' Coverage is established in the AMPM, not the fee schedule, and AHCCCS contractor plans apply their own prior authorization. No AMPM section names 64772, BUT all three UHC Community Plan AZ PA lists state "Experimental and investigational services are not covered benefits" and require PA for any service considered E/I (AMPM 320-B). Combined with CS001.T (endoscopic rhizotomy unproven), an endoscopic MBT is not a covered AHCCCS benefit. AMPM Exhibit 300-1: moderate sedation given by the physician performing the procedure is NOT covered. Fee schedule file is "Effective 7/01/2026" (64772 rate date 10/1/2025). PA phone: ACC/DD 800-445-1638; ALTCS 877-842-3210. Every rendering provider must be AHCCCS-registered. UHC Community Plan policy CS001.T (Arizona is not on its state-exclusion list) lists endoscopic RFA / endoscopic rhizotomy, pulsed, cooled, chemical, laser and cryoablation as unproven and not medically necessary.</t>
+          <t>64772 'TRANSECTION OR AVULSION OF OTHER SPINAL NERVE, EXTRADURAL' at $578.79 non-facility AND facility (rate parity); lower tier $405.15. 64999 is 'BR - by report'. COVERAGE CAVEAT, verbatim: 'the appearance on this website of a code and rate is not an indication of coverage, nor a guarantee of payment.' Coverage is established in the AMPM, not the fee schedule, and AHCCCS contractor plans apply their own prior authorization. No AMPM section names 64772, BUT all three UHC Community Plan AZ PA lists state "Experimental and investigational services are not covered benefits" and require PA for any service considered E/I (AMPM 320-B). Combined with CS001.T (endoscopic rhizotomy unproven), an endoscopic MBT is not a covered AHCCCS benefit. AMPM Exhibit 300-1: moderate sedation given by the physician performing the procedure is NOT covered. Fee schedule file is "Effective 7/01/2026" (64772 rate date 10/1/2025). PA phone: ACC/DD 800-445-1638; ALTCS 877-842-3210. Every rendering provider must be AHCCCS-registered. UHC Community Plan policy CS001.T (Arizona is not on its state-exclusion list) lists endoscopic RFA / endoscopic rhizotomy, pulsed, cooled, chemical, laser and cryoablation as unproven and not medically necessary. KidsCare: no separate KidsCare PA list is on file - confirm which list UHC applies.</t>
         </is>
       </c>
       <c r="U13" s="3" t="inlineStr">
@@ -7379,7 +7379,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Surest (formerly BIND), UMR / UHSS, UHC Level Funded, UnitedHealthOne (Golden Rule grp 705214), Student Resources, Empire Plan, Sierra / Health Plan of Nevada</t>
+          <t>UMR / UHSS, UHC Level Funded, UnitedHealthOne (Golden Rule grp 705214), Student Resources, Empire Plan, Sierra / Health Plan of Nevada</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>For self-funded and level-funded groups the SPD governs the benefit and the TPA's criteria set governs medical necessity, so the answer varies BY GROUP and cannot be resolved at network level. Surest runs a different benefit and PA model from standard UHC Commercial. Empire Plan has an Arizona concentration. SUREST: 64772 is not on the Surest PA list (PCA-1-24-01406, eff. 1 Sep 2026) - Surest itself is NO; the rest of this row stays TO CONFIRM by group.</t>
+          <t>For self-funded and level-funded groups the SPD governs the benefit and the TPA's criteria set governs medical necessity, so the answer varies BY GROUP and cannot be resolved at network level. Empire Plan has an Arizona concentration. Surest now has its own row (own PA list).</t>
         </is>
       </c>
       <c r="U14" s="3" t="inlineStr">
@@ -7680,8 +7680,404 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Complete</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Gated (referral required)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare internal UM</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>NO - not on list</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Prior authorization requirements for UnitedHealthcare Complete</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>PCA-1-25-02057-Clinical-QRG_09172025</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain management section includes 64490, 64493, 64633, 64635. ALL unlisted codes incl. 64999 require PA</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="inlineStr">
+        <is>
+          <t>Ablative Treatment for Spinal Pain; Facet Joint and MBB; Office-Based Procedures - Site of Service; Outpatient Surgical - Site of Service</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>2026T0107II; 2026T0004WW; MP.12.22 (not in repo); MP.11.27 (not in repo)</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>1 Feb 2026; 10 Sep 2026; 1 Jul 2026; 1 Aug 2026</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>NO - absent from all four</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>64772 is not on the UHC Complete list. Members have no non-emergent out-of-network coverage and no coverage outside the service area. Gated plan: electronic PCP referral required before the specialist visit (2026 UHC Administrative Guide). If the procedure is billed as 64999, PA is required. Coverage policy: commercial Ablative Treatment for Spinal Pain (2026T0107II) - endoscopic RFA/rhizotomy unproven.</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>6 / MAI 3 per CMS; this payer may apply its own unit edits</t>
+        </is>
+      </c>
+      <c r="V17" s="3" t="inlineStr">
+        <is>
+          <t>Header note on 2026T0107II: 'Conventional (Thermal) Radiofrequency Ablation requires site of service review.' MP.12.22 covers 64633/64635 but not 64772; it allows ASC only for named exceptions and EXPRESSLY excludes 'surgeon-preferred or proprietary instruments' as justification. NOTE: MP.12.22 and MP.11.27 are not in this repository - their numbers and dates were not re-verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Surest (formerly Bind) / Surest Flex</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Surest</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare (Surest)</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>NO - not on list</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>UHC Provider Portal PA&amp;N tool, or 877-842-3210</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Prior Authorization Requirements for Surest</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>PCA-1-24-01406-Clinical-QRG_05202024</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>NO - absent. No facet codes on this list; pain management = 62320-62327, 62350-62362, 64451, 64484, 64520, 64620, 64640, E0782-E0786</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>Ablative Treatment for Spinal Pain; Facet Joint and MBB; Office-Based Procedures - Site of Service; Outpatient Surgical - Site of Service</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>2026T0107II; 2026T0004WW; MP.12.22 (not in repo); MP.11.27 (not in repo)</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>1 Feb 2026; 10 Sep 2026; 1 Jul 2026; 1 Aug 2026</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>NO - absent from all four</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>64772 is not on the Surest list and is not a Surest Flex "flexible coverage activation" service (activation must be done &gt;=3 business days before the listed services). Coverage policy: commercial Ablative Treatment for Spinal Pain (2026T0107II) - endoscopic RFA/rhizotomy unproven.</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
+          <t>6 / MAI 3 per CMS; this payer may apply its own unit edits</t>
+        </is>
+      </c>
+      <c r="V18" s="3" t="inlineStr">
+        <is>
+          <t>Header note on 2026T0107II: 'Conventional (Thermal) Radiofrequency Ablation requires site of service review.' MP.12.22 covers 64633/64635 but not 64772; it allows ASC only for named exceptions and EXPRESSLY excludes 'surgeon-preferred or proprietary instruments' as justification. NOTE: MP.12.22 and MP.11.27 are not in this repository - their numbers and dates were not re-verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>UHC Community Plan - Developmental Disabilities (DD, incl. DD-CRS)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Medicaid (AHCCCS) - Medicaid and separate-supplement books</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Medicaid</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Community Plan</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>NO - not on list</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>UHC Provider Portal PA&amp;N tool, or 800-445-1638</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Prior authorization requirements for Arizona Developmental Disabilities - UnitedHealthcare Community Plan of Arizona</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>PCA-2-24-03748-Clinical-QRG_12302024</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>NO - absent. 64490 and 64493 require PA (pain injections &amp; management)</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>NO for 64772; endoscopic rhizotomy is UNPROVEN under CS001.T</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>UHC Community Plan Ablative Treatment for Spinal Pain; AHCCCS AMPM 320-B (experimental services); AMPM Exhibit 300-1 (covered services with limitations)</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>CS001.T; AMPM 320-B; AMPM Exhibit 300-1</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>CS001.T eff. 03/01/2026; 320-B eff. 10/01/2022; Exh. 300-1 rev. 07/09/2026</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>NO - 64772 is not named in CS001.T or the AMPM (it appears only on the AHCCCS FFS fee schedule, which is not a coverage document)</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
+        <is>
+          <t>64772 'TRANSECTION OR AVULSION OF OTHER SPINAL NERVE, EXTRADURAL' at $578.79 non-facility AND facility (rate parity); lower tier $405.15. 64999 is 'BR - by report'. COVERAGE CAVEAT, verbatim: 'the appearance on this website of a code and rate is not an indication of coverage, nor a guarantee of payment.' Coverage is established in the AMPM, not the fee schedule, and AHCCCS contractor plans apply their own prior authorization. No AMPM section names 64772, BUT all three UHC Community Plan AZ PA lists state "Experimental and investigational services are not covered benefits" and require PA for any service considered E/I (AMPM 320-B). Combined with CS001.T (endoscopic rhizotomy unproven), an endoscopic MBT is not a covered AHCCCS benefit. AMPM Exhibit 300-1: moderate sedation given by the physician performing the procedure is NOT covered. Fee schedule file is "Effective 7/01/2026" (64772 rate date 10/1/2025). PA phone: ACC/DD 800-445-1638; ALTCS 877-842-3210. Every rendering provider must be AHCCCS-registered. UHC Community Plan policy CS001.T (Arizona is not on its state-exclusion list) lists endoscopic RFA / endoscopic rhizotomy, pulsed, cooled, chemical, laser and cryoablation as unproven and not medically necessary.</t>
+        </is>
+      </c>
+      <c r="U19" s="3" t="inlineStr">
+        <is>
+          <t>6 / MAI 3 (CMS); AHCCCS applies its own edits</t>
+        </is>
+      </c>
+      <c r="V19" s="3" t="inlineStr">
+        <is>
+          <t>AHCCCS publishes a NON-FACILITY rate where Medicare shows NA - the office is theoretically payable on AHCCCS but not on Medicare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>UHC Community Plan - Arizona Long Term Care (ALTCS-EPD)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Medicaid (AHCCCS) - Medicaid and separate-supplement books</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Medicaid</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Community Plan</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>NO - not on list</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>UHC Provider Portal PA&amp;N tool, or 877-842-3210</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Prior authorization requirements for Arizona Long Term Care - UnitedHealthcare Community Plan of Arizona</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>PCA-1-24-03748-Clinical-QRG_12302024</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>NO - absent. 64490 and 64493 require PA (pain injections &amp; management)</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>NO for 64772; endoscopic rhizotomy is UNPROVEN under CS001.T</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>UHC Community Plan Ablative Treatment for Spinal Pain; AHCCCS AMPM 320-B (experimental services); AMPM Exhibit 300-1 (covered services with limitations)</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>CS001.T; AMPM 320-B; AMPM Exhibit 300-1</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>CS001.T eff. 03/01/2026; 320-B eff. 10/01/2022; Exh. 300-1 rev. 07/09/2026</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>NO - 64772 is not named in CS001.T or the AMPM (it appears only on the AHCCCS FFS fee schedule, which is not a coverage document)</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>64772 'TRANSECTION OR AVULSION OF OTHER SPINAL NERVE, EXTRADURAL' at $578.79 non-facility AND facility (rate parity); lower tier $405.15. 64999 is 'BR - by report'. COVERAGE CAVEAT, verbatim: 'the appearance on this website of a code and rate is not an indication of coverage, nor a guarantee of payment.' Coverage is established in the AMPM, not the fee schedule, and AHCCCS contractor plans apply their own prior authorization. No AMPM section names 64772, BUT all three UHC Community Plan AZ PA lists state "Experimental and investigational services are not covered benefits" and require PA for any service considered E/I (AMPM 320-B). Combined with CS001.T (endoscopic rhizotomy unproven), an endoscopic MBT is not a covered AHCCCS benefit. AMPM Exhibit 300-1: moderate sedation given by the physician performing the procedure is NOT covered. Fee schedule file is "Effective 7/01/2026" (64772 rate date 10/1/2025). PA phone: ACC/DD 800-445-1638; ALTCS 877-842-3210. Every rendering provider must be AHCCCS-registered. UHC Community Plan policy CS001.T (Arizona is not on its state-exclusion list) lists endoscopic RFA / endoscopic rhizotomy, pulsed, cooled, chemical, laser and cryoablation as unproven and not medically necessary.</t>
+        </is>
+      </c>
+      <c r="U20" s="3" t="inlineStr">
+        <is>
+          <t>6 / MAI 3 (CMS); AHCCCS applies its own edits</t>
+        </is>
+      </c>
+      <c r="V20" s="3" t="inlineStr">
+        <is>
+          <t>AHCCCS publishes a NON-FACILITY rate where Medicare shows NA - the office is theoretically payable on AHCCCS but not on Medicare.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V16"/>
+  <autoFilter ref="A1:V20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9032,22 +9428,22 @@
       </c>
       <c r="K9" s="10" t="inlineStr">
         <is>
-          <t>None - the Humana PA list states Medicare Supplement plans are not subject to it</t>
+          <t>None - Medicare Supplement is not subject to prior authorization</t>
         </is>
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>790807ALL0725-C GHHMXVMEN (exclusion note)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
         <is>
-          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N9" s="10" t="inlineStr">
         <is>
-          <t>n/a - Medicare Supplement is excluded from the list</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="O9" s="10" t="inlineStr">
@@ -9077,7 +9473,7 @@
       </c>
       <c r="T9" s="10" t="inlineStr">
         <is>
-          <t>No PA. Humana Medigap pays after Medicare's decision - if Medicare denies on review, Humana pays nothing. NAME CHECK: HumanaMS.pdf (Maricopa 85023 plan list) names the plans "Humana Plan F", "Humana Plan N" etc.; the labels "VALUE" / "ACHIEVE" do not appear in any repository document - confirm against the member card.</t>
+          <t>No PA. Humana Medigap pays after Medicare's decision - if Medicare denies on review, Humana pays nothing. NAME CHECK: HumanaMS.pdf (Maricopa 85023 plan list) names the plans "Humana Plan F", "Humana Plan N" etc.; the labels "VALUE" / "ACHIEVE" do not appear in any repository document - confirm against the member card. (The Humana MA/D-SNP PA list 790807ALL0725-C states it "does not apply to policy holders of a Humana Medicare Supplement plan".)</t>
         </is>
       </c>
       <c r="U9" s="10" t="inlineStr">
@@ -9144,22 +9540,22 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>None - the Humana PA list states Medicare Supplement plans are not subject to it</t>
+          <t>None - Medicare Supplement is not subject to prior authorization</t>
         </is>
       </c>
       <c r="L10" s="10" t="inlineStr">
         <is>
-          <t>790807ALL0725-C GHHMXVMEN (exclusion note)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N10" s="10" t="inlineStr">
         <is>
-          <t>n/a - Medicare Supplement is excluded from the list</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -9256,22 +9652,22 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>None - the Humana PA list states Medicare Supplement plans are not subject to it</t>
+          <t>None - Medicare Supplement is not subject to prior authorization</t>
         </is>
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>790807ALL0725-C GHHMXVMEN (exclusion note)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
+          <t>-</t>
         </is>
       </c>
       <c r="N11" s="10" t="inlineStr">
         <is>
-          <t>n/a - Medicare Supplement is excluded from the list</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -9606,7 +10002,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -10740,7 +11135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D877"/>
+  <dimension ref="A1:D982"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -29803,6 +30198,2263 @@
         </is>
       </c>
     </row>
+    <row r="879">
+      <c r="A879" s="15" t="inlineStr">
+        <is>
+          <t>Round 4 - PA documents re-matched to the correct payer/plan (user correction), 23 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B880" s="17" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="C880" s="17" t="inlineStr">
+        <is>
+          <t>Navigate, Charter, Compass, NexusACO R / RB / RP, Freedom Granite Advantage-Saver EPO, UHC Complete</t>
+        </is>
+      </c>
+      <c r="D880" s="17" t="inlineStr">
+        <is>
+          <t>Navigate, Charter, Compass, NexusACO R / RB / RP, Freedom Granite Advantage-Saver EPO</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B881" s="17" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="C881" s="17" t="inlineStr">
+        <is>
+          <t>64772 is absent from all four. But related techniques are AFFIRMATIVELY unproven and not medically necessary: pulsed RFA, endoscopic RFA / endoscopic rhizotomy, cryoablation, cooled RFA, chemical ablation, laser ablation. 'Ablation for treating sacroiliac pain is unproven and not medically necessary' - so 64625 is not covered commercially. Facet diagnostic block covered only when: facet loading pain on exam; no significant improvement (pain still &gt;=3/10) after &gt;=4 weeks conservative care; imaging excludes other causes; segment not fused; AND an RFA is being considered. Absence from a policy is</t>
+        </is>
+      </c>
+      <c r="D881" s="17" t="inlineStr">
+        <is>
+          <t>64772 is absent from all four. But related techniques are AFFIRMATIVELY unproven and not medically necessary: pulsed RFA, endoscopic RFA / endoscopic rhizotomy, cryoablation, cooled RFA, chemical ablation, laser ablation. 'Ablation for treating sacroiliac pain is unproven and not medically necessary' - so 64625 is not covered commercially. Facet diagnostic block covered only when: facet loading pain on exam; no significant improvement (pain still &gt;=3/10) after &gt;=4 weeks conservative care; imaging excludes other causes; segment not fused; AND an RFA is being considered. Absence from a policy is</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B882" s="17" t="inlineStr">
+        <is>
+          <t>A17:V17</t>
+        </is>
+      </c>
+      <c r="C882" s="17" t="inlineStr"/>
+      <c r="D882" s="17" t="inlineStr">
+        <is>
+          <t>NEW ROW: UnitedHealthcare Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B883" s="17" t="inlineStr">
+        <is>
+          <t>A14</t>
+        </is>
+      </c>
+      <c r="C883" s="17" t="inlineStr">
+        <is>
+          <t>Surest (formerly BIND), UMR / UHSS, UHC Level Funded, UnitedHealthOne (Golden Rule grp 705214), Student Resources, Empire Plan, Sierra / Health Plan of Nevada</t>
+        </is>
+      </c>
+      <c r="D883" s="17" t="inlineStr">
+        <is>
+          <t>UMR / UHSS, UHC Level Funded, UnitedHealthOne (Golden Rule grp 705214), Student Resources, Empire Plan, Sierra / Health Plan of Nevada</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B884" s="17" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C884" s="17" t="inlineStr">
+        <is>
+          <t>For self-funded and level-funded groups the SPD governs the benefit and the TPA's criteria set governs medical necessity, so the answer varies BY GROUP and cannot be resolved at network level. Surest runs a different benefit and PA model from standard UHC Commercial. Empire Plan has an Arizona concentration. SUREST: 64772 is not on the Surest PA list (PCA-1-24-01406, eff. 1 Sep 2026) - Surest itself is NO; the rest of this row stays TO CONFIRM by group.</t>
+        </is>
+      </c>
+      <c r="D884" s="17" t="inlineStr">
+        <is>
+          <t>For self-funded and level-funded groups the SPD governs the benefit and the TPA's criteria set governs medical necessity, so the answer varies BY GROUP and cannot be resolved at network level. Empire Plan has an Arizona concentration. Surest now has its own row (own PA list).</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B885" s="17" t="inlineStr">
+        <is>
+          <t>A18:V18</t>
+        </is>
+      </c>
+      <c r="C885" s="17" t="inlineStr"/>
+      <c r="D885" s="17" t="inlineStr">
+        <is>
+          <t>NEW ROW: Surest (formerly Bind) / Surest Flex</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B886" s="17" t="inlineStr">
+        <is>
+          <t>A13</t>
+        </is>
+      </c>
+      <c r="C886" s="17" t="inlineStr">
+        <is>
+          <t>UHC Community Plan - ACC, ACC-CRS, DD, DD-CRS, KidsCare, ALTCS-EPD</t>
+        </is>
+      </c>
+      <c r="D886" s="17" t="inlineStr">
+        <is>
+          <t>UHC Community Plan - AHCCCS Complete Care (ACC, incl. CRS-designated members)</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B887" s="17" t="inlineStr">
+        <is>
+          <t>K13</t>
+        </is>
+      </c>
+      <c r="C887" s="17" t="inlineStr">
+        <is>
+          <t>UHC Community Plan of AZ PA requirements - ACC, Developmental Disabilities, Long Term Care</t>
+        </is>
+      </c>
+      <c r="D887" s="17" t="inlineStr">
+        <is>
+          <t>Prior authorization requirements for AHCCCS Complete Care (ACC) Medicaid - UnitedHealthcare Community Plan of Arizona</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B888" s="17" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="C888" s="17" t="inlineStr">
+        <is>
+          <t>PCA-5-24-03748 (ACC); PCA-2-24-03748 (DD); PCA-1-24-03748 (ALTCS)</t>
+        </is>
+      </c>
+      <c r="D888" s="17" t="inlineStr">
+        <is>
+          <t>PCA-5-24-003748-Clinical-QRG_05192023</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B889" s="17" t="inlineStr">
+        <is>
+          <t>N13</t>
+        </is>
+      </c>
+      <c r="C889" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from all three. 64490/64493 require PA (pain injections)</t>
+        </is>
+      </c>
+      <c r="D889" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. 64490 and 64493 require PA (pain injections &amp; management)</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B890" s="17" t="inlineStr">
+        <is>
+          <t>J13</t>
+        </is>
+      </c>
+      <c r="C890" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal</t>
+        </is>
+      </c>
+      <c r="D890" s="17" t="inlineStr">
+        <is>
+          <t>UHC Provider Portal PA&amp;N tool, or 800-445-1638</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B891" s="17" t="inlineStr">
+        <is>
+          <t>A19:V19</t>
+        </is>
+      </c>
+      <c r="C891" s="17" t="inlineStr"/>
+      <c r="D891" s="17" t="inlineStr">
+        <is>
+          <t>NEW ROW: UHC Community Plan - Developmental Disabilities (DD, incl. DD-CRS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B892" s="17" t="inlineStr">
+        <is>
+          <t>A20:V20</t>
+        </is>
+      </c>
+      <c r="C892" s="17" t="inlineStr"/>
+      <c r="D892" s="17" t="inlineStr">
+        <is>
+          <t>NEW ROW: UHC Community Plan - Arizona Long Term Care (ALTCS-EPD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B893" s="17" t="inlineStr">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="C893" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D893" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B894" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C894" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D894" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B895" s="17" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="C895" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D895" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B896" s="17" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="C896" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D896" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B897" s="17" t="inlineStr">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="C897" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D897" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B898" s="17" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="C898" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D898" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B899" s="17" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="C899" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D899" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B900" s="17" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C900" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D900" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B901" s="17" t="inlineStr">
+        <is>
+          <t>K4</t>
+        </is>
+      </c>
+      <c r="C901" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D901" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B902" s="17" t="inlineStr">
+        <is>
+          <t>L4</t>
+        </is>
+      </c>
+      <c r="C902" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D902" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B903" s="17" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="C903" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D903" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B904" s="17" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="C904" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D904" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B905" s="17" t="inlineStr">
+        <is>
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="C905" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D905" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B906" s="17" t="inlineStr">
+        <is>
+          <t>L5</t>
+        </is>
+      </c>
+      <c r="C906" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D906" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B907" s="17" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="C907" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D907" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B908" s="17" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="C908" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D908" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B909" s="17" t="inlineStr">
+        <is>
+          <t>K6</t>
+        </is>
+      </c>
+      <c r="C909" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D909" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B910" s="17" t="inlineStr">
+        <is>
+          <t>L6</t>
+        </is>
+      </c>
+      <c r="C910" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D910" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B911" s="17" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="C911" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D911" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B912" s="17" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="C912" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D912" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B913" s="17" t="inlineStr">
+        <is>
+          <t>K7</t>
+        </is>
+      </c>
+      <c r="C913" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D913" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B914" s="17" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="C914" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D914" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B915" s="17" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="C915" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D915" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B916" s="17" t="inlineStr">
+        <is>
+          <t>N7</t>
+        </is>
+      </c>
+      <c r="C916" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D916" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B917" s="17" t="inlineStr">
+        <is>
+          <t>K8</t>
+        </is>
+      </c>
+      <c r="C917" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D917" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B918" s="17" t="inlineStr">
+        <is>
+          <t>L8</t>
+        </is>
+      </c>
+      <c r="C918" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D918" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B919" s="17" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="C919" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D919" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B920" s="17" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="C920" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D920" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B921" s="17" t="inlineStr">
+        <is>
+          <t>K9</t>
+        </is>
+      </c>
+      <c r="C921" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D921" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B922" s="17" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
+      <c r="C922" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D922" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B923" s="17" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="C923" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D923" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B924" s="17" t="inlineStr">
+        <is>
+          <t>N9</t>
+        </is>
+      </c>
+      <c r="C924" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D924" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B925" s="17" t="inlineStr">
+        <is>
+          <t>K10</t>
+        </is>
+      </c>
+      <c r="C925" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D925" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B926" s="17" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="C926" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D926" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B927" s="17" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="C927" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D927" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B928" s="17" t="inlineStr">
+        <is>
+          <t>N10</t>
+        </is>
+      </c>
+      <c r="C928" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D928" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B929" s="17" t="inlineStr">
+        <is>
+          <t>K11</t>
+        </is>
+      </c>
+      <c r="C929" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D929" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B930" s="17" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="C930" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D930" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B931" s="17" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="C931" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D931" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B932" s="17" t="inlineStr">
+        <is>
+          <t>N11</t>
+        </is>
+      </c>
+      <c r="C932" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D932" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B933" s="17" t="inlineStr">
+        <is>
+          <t>K12</t>
+        </is>
+      </c>
+      <c r="C933" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D933" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B934" s="17" t="inlineStr">
+        <is>
+          <t>L12</t>
+        </is>
+      </c>
+      <c r="C934" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D934" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B935" s="17" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="C935" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D935" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B936" s="17" t="inlineStr">
+        <is>
+          <t>N12</t>
+        </is>
+      </c>
+      <c r="C936" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D936" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B937" s="17" t="inlineStr">
+        <is>
+          <t>K13</t>
+        </is>
+      </c>
+      <c r="C937" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D937" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B938" s="17" t="inlineStr">
+        <is>
+          <t>L13</t>
+        </is>
+      </c>
+      <c r="C938" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D938" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B939" s="17" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="C939" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D939" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B940" s="17" t="inlineStr">
+        <is>
+          <t>N13</t>
+        </is>
+      </c>
+      <c r="C940" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D940" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B941" s="17" t="inlineStr">
+        <is>
+          <t>K14</t>
+        </is>
+      </c>
+      <c r="C941" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: UHC Medicare Advantage prior authorization and referral requirements</t>
+        </is>
+      </c>
+      <c r="D941" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona UHC MA PA and referral requirements. All other providers: UHC Medicare Advantage PA requirements (per the Optum list header and UHC/Optum QRG PCA-4-26-00582)</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B942" s="17" t="inlineStr">
+        <is>
+          <t>L14</t>
+        </is>
+      </c>
+      <c r="C942" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026</t>
+        </is>
+      </c>
+      <c r="D942" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928_08262026 (Optum-direct); PCA-4-26-00416-Clinical-QRG_03022026 (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B943" s="17" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="C943" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D943" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 1 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B944" s="17" t="inlineStr">
+        <is>
+          <t>N14</t>
+        </is>
+      </c>
+      <c r="C944" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent. Pain Management lists 0627T-0630T, 62350-62362, 64490-64495, 64628/64629, 64633-64636</t>
+        </is>
+      </c>
+      <c r="D944" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B945" s="17" t="inlineStr">
+        <is>
+          <t>K15</t>
+        </is>
+      </c>
+      <c r="C945" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+        </is>
+      </c>
+      <c r="D945" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B946" s="17" t="inlineStr">
+        <is>
+          <t>L15</t>
+        </is>
+      </c>
+      <c r="C946" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026</t>
+        </is>
+      </c>
+      <c r="D946" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B947" s="17" t="inlineStr">
+        <is>
+          <t>M15</t>
+        </is>
+      </c>
+      <c r="C947" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D947" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B948" s="17" t="inlineStr">
+        <is>
+          <t>N15</t>
+        </is>
+      </c>
+      <c r="C948" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent (facet family is listed)</t>
+        </is>
+      </c>
+      <c r="D948" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B949" s="17" t="inlineStr">
+        <is>
+          <t>K16</t>
+        </is>
+      </c>
+      <c r="C949" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+        </is>
+      </c>
+      <c r="D949" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B950" s="17" t="inlineStr">
+        <is>
+          <t>L16</t>
+        </is>
+      </c>
+      <c r="C950" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026</t>
+        </is>
+      </c>
+      <c r="D950" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B951" s="17" t="inlineStr">
+        <is>
+          <t>M16</t>
+        </is>
+      </c>
+      <c r="C951" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D951" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B952" s="17" t="inlineStr">
+        <is>
+          <t>N16</t>
+        </is>
+      </c>
+      <c r="C952" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent (facet family is listed)</t>
+        </is>
+      </c>
+      <c r="D952" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B953" s="17" t="inlineStr">
+        <is>
+          <t>K8</t>
+        </is>
+      </c>
+      <c r="C953" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+        </is>
+      </c>
+      <c r="D953" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B954" s="17" t="inlineStr">
+        <is>
+          <t>L8</t>
+        </is>
+      </c>
+      <c r="C954" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026</t>
+        </is>
+      </c>
+      <c r="D954" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B955" s="17" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="C955" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D955" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B956" s="17" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="C956" s="17" t="inlineStr">
+        <is>
+          <t>NO - not listed. Pain Management section lists 62350-62362, 64490-64495, 64628/64629, 64633-64636 - not 64772</t>
+        </is>
+      </c>
+      <c r="D956" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B957" s="17" t="inlineStr">
+        <is>
+          <t>K10</t>
+        </is>
+      </c>
+      <c r="C957" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+        </is>
+      </c>
+      <c r="D957" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B958" s="17" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="C958" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026</t>
+        </is>
+      </c>
+      <c r="D958" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B959" s="17" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="C959" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D959" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B960" s="17" t="inlineStr">
+        <is>
+          <t>N10</t>
+        </is>
+      </c>
+      <c r="C960" s="17" t="inlineStr">
+        <is>
+          <t>NO - not listed (facet family 64490-64495 / 64633-64636 is listed)</t>
+        </is>
+      </c>
+      <c r="D960" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B961" s="17" t="inlineStr">
+        <is>
+          <t>K11</t>
+        </is>
+      </c>
+      <c r="C961" s="17" t="inlineStr">
+        <is>
+          <t>2026 OptumCare Network of Arizona: Blue Cross Blue Shield prior authorization requirements</t>
+        </is>
+      </c>
+      <c r="D961" s="17" t="inlineStr">
+        <is>
+          <t>Optum-DIRECT contracted providers: 2026 OptumCare Network of Arizona BCBS PA requirements. All other providers: AZ Blue 2026 Medicare Advantage List (per the Optum list header)</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B962" s="17" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="C962" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026</t>
+        </is>
+      </c>
+      <c r="D962" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00929_09032026 (Optum-direct); AZ Blue 2026 Medicare Advantage List (all others)</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B963" s="17" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="C963" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, updated 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D963" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jan 2026, upd. 1 Sep 2026; Eff. 09/01/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B964" s="17" t="inlineStr">
+        <is>
+          <t>N11</t>
+        </is>
+      </c>
+      <c r="C964" s="17" t="inlineStr">
+        <is>
+          <t>NO - not listed (facet family 64490-64495 / 64633-64636 is listed)</t>
+        </is>
+      </c>
+      <c r="D964" s="17" t="inlineStr">
+        <is>
+          <t>NO - absent from both lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B965" s="17" t="inlineStr">
+        <is>
+          <t>K9</t>
+        </is>
+      </c>
+      <c r="C965" s="17" t="inlineStr">
+        <is>
+          <t>None - the Humana PA list states Medicare Supplement plans are not subject to it</t>
+        </is>
+      </c>
+      <c r="D965" s="17" t="inlineStr">
+        <is>
+          <t>None - Medicare Supplement is not subject to prior authorization</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B966" s="17" t="inlineStr">
+        <is>
+          <t>L9</t>
+        </is>
+      </c>
+      <c r="C966" s="17" t="inlineStr">
+        <is>
+          <t>790807ALL0725-C GHHMXVMEN (exclusion note)</t>
+        </is>
+      </c>
+      <c r="D966" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B967" s="17" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="C967" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D967" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B968" s="17" t="inlineStr">
+        <is>
+          <t>N9</t>
+        </is>
+      </c>
+      <c r="C968" s="17" t="inlineStr">
+        <is>
+          <t>n/a - Medicare Supplement is excluded from the list</t>
+        </is>
+      </c>
+      <c r="D968" s="17" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B969" s="17" t="inlineStr">
+        <is>
+          <t>K10</t>
+        </is>
+      </c>
+      <c r="C969" s="17" t="inlineStr">
+        <is>
+          <t>None - the Humana PA list states Medicare Supplement plans are not subject to it</t>
+        </is>
+      </c>
+      <c r="D969" s="17" t="inlineStr">
+        <is>
+          <t>None - Medicare Supplement is not subject to prior authorization</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B970" s="17" t="inlineStr">
+        <is>
+          <t>L10</t>
+        </is>
+      </c>
+      <c r="C970" s="17" t="inlineStr">
+        <is>
+          <t>790807ALL0725-C GHHMXVMEN (exclusion note)</t>
+        </is>
+      </c>
+      <c r="D970" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B971" s="17" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="C971" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D971" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B972" s="17" t="inlineStr">
+        <is>
+          <t>N10</t>
+        </is>
+      </c>
+      <c r="C972" s="17" t="inlineStr">
+        <is>
+          <t>n/a - Medicare Supplement is excluded from the list</t>
+        </is>
+      </c>
+      <c r="D972" s="17" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B973" s="17" t="inlineStr">
+        <is>
+          <t>K11</t>
+        </is>
+      </c>
+      <c r="C973" s="17" t="inlineStr">
+        <is>
+          <t>None - the Humana PA list states Medicare Supplement plans are not subject to it</t>
+        </is>
+      </c>
+      <c r="D973" s="17" t="inlineStr">
+        <is>
+          <t>None - Medicare Supplement is not subject to prior authorization</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B974" s="17" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="C974" s="17" t="inlineStr">
+        <is>
+          <t>790807ALL0725-C GHHMXVMEN (exclusion note)</t>
+        </is>
+      </c>
+      <c r="D974" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B975" s="17" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="C975" s="17" t="inlineStr">
+        <is>
+          <t>Eff. 1 Jul 2026, rev. 1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="D975" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B976" s="17" t="inlineStr">
+        <is>
+          <t>N11</t>
+        </is>
+      </c>
+      <c r="C976" s="17" t="inlineStr">
+        <is>
+          <t>n/a - Medicare Supplement is excluded from the list</t>
+        </is>
+      </c>
+      <c r="D976" s="17" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B977" s="17" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="C977" s="17" t="inlineStr">
+        <is>
+          <t>No PA. Humana Medigap pays after Medicare's decision - if Medicare denies on review, Humana pays nothing. NAME CHECK: HumanaMS.pdf (Maricopa 85023 plan list) names the plans "Humana Plan F", "Humana Plan N" etc.; the labels "VALUE" / "ACHIEVE" do not appear in any repository document - confirm against the member card.</t>
+        </is>
+      </c>
+      <c r="D977" s="17" t="inlineStr">
+        <is>
+          <t>No PA. Humana Medigap pays after Medicare's decision - if Medicare denies on review, Humana pays nothing. NAME CHECK: HumanaMS.pdf (Maricopa 85023 plan list) names the plans "Humana Plan F", "Humana Plan N" etc.; the labels "VALUE" / "ACHIEVE" do not appear in any repository document - confirm against the member card. (The Humana MA/D-SNP PA list 790807ALL0725-C states it "does not apply to policy holders of a Humana Medicare Supplement plan".)</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B978" s="17" t="inlineStr">
+        <is>
+          <t>B16</t>
+        </is>
+      </c>
+      <c r="C978" s="17" t="inlineStr">
+        <is>
+          <t>AZ Blue MA list 09/01/2026; Optum BCBS list OHNC-1-25-00929</t>
+        </is>
+      </c>
+      <c r="D978" s="17" t="inlineStr">
+        <is>
+          <t>AZ Blue MA list 09/01/2026; Optum BCBS list OHNC-1-25-00929 only for Optum-direct providers</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B979" s="17" t="inlineStr">
+        <is>
+          <t>B19</t>
+        </is>
+      </c>
+      <c r="C979" s="17" t="inlineStr">
+        <is>
+          <t>None (excluded from Humana PA list); Medicare decides</t>
+        </is>
+      </c>
+      <c r="D979" s="17" t="inlineStr">
+        <is>
+          <t>None - not subject to PA; Medicare decides</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B980" s="17" t="inlineStr">
+        <is>
+          <t>B21</t>
+        </is>
+      </c>
+      <c r="C980" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928 (eff. 1 Jan 2026, upd. 1 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="D980" s="17" t="inlineStr">
+        <is>
+          <t>OHNC-1-25-00928 if Optum-direct; otherwise UHC MA list PCA-4-26-00416</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B981" s="17" t="inlineStr">
+        <is>
+          <t>B22</t>
+        </is>
+      </c>
+      <c r="C981" s="17" t="inlineStr">
+        <is>
+          <t>PCA-1-26-00657; PCA-5-26-00416; 2026T0107II</t>
+        </is>
+      </c>
+      <c r="D981" s="17" t="inlineStr">
+        <is>
+          <t>PCA-1-26-00657 (Commercial); PCA-5-26-00416 (Exchange); PCA-1-25-02057 (UHC Complete); PCA-1-24-01406 (Surest); 2026T0107II</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B982" s="17" t="inlineStr">
+        <is>
+          <t>B23</t>
+        </is>
+      </c>
+      <c r="C982" s="17" t="inlineStr">
+        <is>
+          <t>PCA-x-24-03748; CS001.T; PCA-4-26-00416</t>
+        </is>
+      </c>
+      <c r="D982" s="17" t="inlineStr">
+        <is>
+          <t>ACC PCA-5-24-003748; DD PCA-2-24-03748; ALTCS PCA-1-24-03748; Dual Complete PCA-4-26-00416; CS001.T</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove referral information from the 64772 routing workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiByUV3Zo1mhZNaeehe8GC
</commit_message>
<xml_diff>
--- a/Code Research/CPT_64772_Routing_2026.xlsx
+++ b/Code Research/CPT_64772_Routing_2026.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -602,6 +602,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -651,6 +652,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -900,7 +902,7 @@
       </c>
       <c r="D20" s="17" t="inlineStr">
         <is>
-          <t>Follows NCD 160.1 / L38801 (endoscopic evidence "insufficient"); commercial Ablative policy (endoscopic = unproven) may fill gaps. HMO/HMO-POS (incl. D-SNP/C-SNP HMO): PCP referral required.</t>
+          <t>Follows NCD 160.1 / L38801 (endoscopic evidence "insufficient"); UHC commercial policy calls endoscopic rhizotomy unproven.</t>
         </is>
       </c>
       <c r="E20" s="17" t="inlineStr">
@@ -932,12 +934,12 @@
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>HMO/HMO-POS: PCP referral to Optum required before the visit (except H5253-035, I-SNP, Erickson).</t>
+          <t>Same coverage position as UHC MA (NCD 160.1 / L38801).</t>
         </is>
       </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
-          <t>Referral on file</t>
+          <t>Pre-service decision on optumproportal.com if endoscopic</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -964,7 +966,7 @@
       </c>
       <c r="D22" s="17" t="inlineStr">
         <is>
-          <t>Endoscopic RFA/rhizotomy UNPROVEN. AZ Pain Management Program: 64490-64495 PA in all places of service. Gated plans need an electronic PCP referral; the AZ Exchange needs a PCP referral before any PA.</t>
+          <t>Endoscopic RFA/rhizotomy UNPROVEN (2026T0107II). AZ Pain Management Program: 64490-64495 need PA in all places of service.</t>
         </is>
       </c>
       <c r="E22" s="17" t="inlineStr">
@@ -1234,79 +1236,74 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>[ ] Referral on file where the plan requires one (UHC MA HMO/HMO-POS incl. D-SNP/C-SNP, Optum-delegated HMO - PCP submits it; UHC gated commercial; UHC AZ Exchange; Dual Complete).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="28" customHeight="1"/>
+    <row r="39" ht="30" customHeight="1"/>
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+    </row>
     <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="15" t="inlineStr">
-        <is>
-          <t>Open items</t>
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>- SCAN (Optum-delegated): call Optum 877-370-2845 once to confirm no auth; record the reference #.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>- SCAN (Optum-delegated): call Optum 877-370-2845 once to confirm no auth; record the reference #.</t>
+          <t>- AZ Blue: resolve the IVR prefix conflict (Strategic Hub vs Standard list); get a written predetermination for the first case.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>- AZ Blue: resolve the IVR prefix conflict (Strategic Hub vs Standard list); get a written predetermination for the first case.</t>
+          <t>- TPA groups (AHG, AmeriBen), BCBS SC, CHS, BlueCard home plans, Banner, delegated IPAs: call and record.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>- TPA groups (AHG, AmeriBen), BCBS SC, CHS, BlueCard home plans, Banner, delegated IPAs: call and record.</t>
+          <t>- AZPC Attachment A and the Health Choice PA grids are not in the repository; those rows rely on your portal checks.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>- AZPC Attachment A and the Health Choice PA grids are not in the repository; those rows rely on your portal checks.</t>
+          <t>- Code selection (64772 vs 64999) for endoscopic MBT: confirm with the coding team from the operative note.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>- Code selection (64772 vs 64999) for endoscopic MBT: confirm with the coding team from the operative note.</t>
+          <t>- Confirm whether Dr. Luke is Optum-direct contracted (the Optum lists apply only to direct contracts).</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>- Confirm whether Dr. Luke is Optum-direct contracted (the Optum lists apply only to direct contracts).</t>
+          <t>- Dr. Luke's procedure claims in 2026 S1 were billed at ASAP Surgery Centers North Valley LLC (ASC); confirm the ASC is contracted with each payer and obtain the ASC's own authorization where the payer requires a facility PA (AHCCCS FFS).</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>- Dr. Luke's procedure claims in 2026 S1 were billed at ASAP Surgery Centers North Valley LLC (ASC); confirm the ASC is contracted with each payer and obtain the ASC's own authorization where the payer requires a facility PA (AHCCCS FFS).</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
           <t>- No 64772, 64999 or facet (64490-64495 / 64633-64636) claims appear in the 2026 S1 claims files - there is no payment history yet; track the first claims per payer closely.</t>
         </is>
       </c>
     </row>
+    <row r="49" ht="30" customHeight="1"/>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="23">
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="A33:F33"/>
@@ -1325,8 +1322,6 @@
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A48:F48"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A49:F49"/>
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="A45:F45"/>
     <mergeCell ref="A6:F6"/>
@@ -3517,9 +3512,8 @@
       <c r="T2" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
@@ -3632,9 +3626,8 @@
       <c r="T3" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -3747,9 +3740,8 @@
       <c r="T4" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: NOT required (H5253-035 is exempt).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -3862,9 +3854,8 @@
       <c r="T5" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -3977,9 +3968,8 @@
       <c r="T6" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -4092,9 +4082,8 @@
       <c r="T7" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -4207,9 +4196,8 @@
       <c r="T8" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
@@ -4322,9 +4310,8 @@
       <c r="T9" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U9" s="3" t="inlineStr">
@@ -4437,9 +4424,8 @@
       <c r="T10" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U10" s="3" t="inlineStr">
@@ -4552,9 +4538,8 @@
       <c r="T11" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: NOT required (PPO).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U11" s="3" t="inlineStr">
@@ -4667,9 +4652,8 @@
       <c r="T12" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: NOT required (PPO).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U12" s="3" t="inlineStr">
@@ -4782,9 +4766,8 @@
       <c r="T13" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: NOT required (PPO).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U13" s="3" t="inlineStr">
@@ -4897,9 +4880,8 @@
       <c r="T14" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
-Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
-Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com.</t>
         </is>
       </c>
       <c r="U14" s="3" t="inlineStr">
@@ -6375,7 +6357,6 @@
       <c r="T2" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
-Referral: REQUIRED - PCP referral on file before the visit (2026 UHC Administrative Guide).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
 Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is endoscopic, request a pre-service organization determination (PA&amp;N tool).</t>
         </is>
@@ -6474,7 +6455,6 @@
       <c r="T3" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
-Referral: REQUIRED - PCP referral on file before the visit (2026 UHC Administrative Guide).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
 Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is endoscopic, request a pre-service organization determination (PA&amp;N tool).</t>
         </is>
@@ -6573,7 +6553,6 @@
       <c r="T4" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
-Referral: NOT required.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
 Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is endoscopic, request a pre-service organization determination (PA&amp;N tool).</t>
         </is>
@@ -6672,7 +6651,6 @@
       <c r="T5" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
-Referral: REQUIRED - PCP referral on file before the visit (2026 UHC Administrative Guide).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
 Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is endoscopic, request a pre-service organization determination (PA&amp;N tool).</t>
         </is>
@@ -6771,7 +6749,6 @@
       <c r="T6" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
-Referral: NOT required.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
 Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is endoscopic, request a pre-service organization determination (PA&amp;N tool).</t>
         </is>
@@ -6870,7 +6847,6 @@
       <c r="T7" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
-Referral: NOT required.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
 Action: if the MBT is endoscopic, call the Erickson PA number on the ID card - Erickson requires PA for experimental/investigational services.</t>
         </is>
@@ -6969,7 +6945,6 @@
       <c r="T8" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either. The list names UHC Dual Complete as included.
-Referral: members must coordinate with their PCP; non-contracted providers need a referral form and PA (Dual Complete manual).
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven. Medicaid wrap: experimental services are not AHCCCS benefits.
 Action: PA line 800-445-1638 if needed. QMB members owe $0 - do not bill the member.</t>
         </is>
@@ -7068,7 +7043,6 @@
       <c r="T9" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
-Referral: NOT required.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
 Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is endoscopic, request a pre-service organization determination (PA&amp;N tool).</t>
         </is>
@@ -7167,7 +7141,6 @@
       <c r="T10" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC Commercial list (eff. 9/1/2026). Arizona Pain Management Program: 64490-64495 need PA in all places of service; 64490/64493/64633/64635 need PA when done in hospital outpatient or ASC.
-Referral: REQUIRED - electronic PCP referral before the visit.
 Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
 Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
         </is>
@@ -7266,7 +7239,6 @@
       <c r="T11" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC Commercial list (eff. 9/1/2026). Arizona Pain Management Program: 64490-64495 need PA in all places of service; 64490/64493/64633/64635 need PA when done in hospital outpatient or ASC.
-Referral: NOT required.
 Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
 Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
         </is>
@@ -7373,7 +7345,6 @@
       <c r="T12" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the Individual Exchange list (eff. 9/1/2026). 64999 WOULD need PA. 64490, 64493, 64633, 64635 need PA + site-of-service review.
-Referral: REQUIRED in Arizona - UHC will not accept a PA without a referral on file. No out-of-network coverage.
 Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
 Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
         </is>
@@ -7807,7 +7778,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Gated (referral required)</t>
+          <t>Gated</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
@@ -7877,7 +7848,6 @@
       <c r="T17" s="3" t="inlineStr">
         <is>
           <t>PA: NOT required - 64772 is not on the UHC Complete list (eff. 9/1/2026). 64999 WOULD need PA.
-Referral: REQUIRED - electronic PCP referral. No out-of-network coverage.
 Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
 Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
         </is>
@@ -11242,7 +11212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1269"/>
+  <dimension ref="A1:D1315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -38971,6 +38941,1147 @@
         </is>
       </c>
     </row>
+    <row r="1271">
+      <c r="A1271" s="15" t="inlineStr">
+        <is>
+          <t>Round 6 - referral information removed (not requested), 23 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1272" s="17" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C1272" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1272" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1273" s="17" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C1273" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1273" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1274" s="17" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C1274" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: NOT required (H5253-035 is exempt).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file;</t>
+        </is>
+      </c>
+      <c r="D1274" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1275" s="17" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C1275" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1275" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1276" s="17" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C1276" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1276" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1277" s="17" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C1277" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1277" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1278" s="17" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="C1278" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1278" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1279" s="17" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="C1279" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1279" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1280" s="17" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="C1280" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1280" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1281" s="17" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="C1281" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: NOT required (PPO).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is e</t>
+        </is>
+      </c>
+      <c r="D1281" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1282" s="17" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="C1282" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: NOT required (PPO).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is e</t>
+        </is>
+      </c>
+      <c r="D1282" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1283" s="17" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="C1283" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: NOT required (PPO).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is e</t>
+        </is>
+      </c>
+      <c r="D1283" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1284" s="17" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C1284" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Referral: REQUIRED - the PCP must submit it to Optum before the visit (orthopaedist and neurosurgeon are listed specialties); no referral = claim denied, provider liability, member cannot be billed.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDO</t>
+        </is>
+      </c>
+      <c r="D1284" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1285" s="17" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C1285" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Referral: REQUIRED - PCP referral on file before the visit (2026 UHC Administrative Guide).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action:</t>
+        </is>
+      </c>
+      <c r="D1285" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1286" s="17" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C1286" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Referral: REQUIRED - PCP referral on file before the visit (2026 UHC Administrative Guide).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action:</t>
+        </is>
+      </c>
+      <c r="D1286" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1287" s="17" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C1287" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Referral: NOT required.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the </t>
+        </is>
+      </c>
+      <c r="D1287" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1288" s="17" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C1288" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Referral: REQUIRED - PCP referral on file before the visit (2026 UHC Administrative Guide).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action:</t>
+        </is>
+      </c>
+      <c r="D1288" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1289" s="17" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C1289" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Referral: NOT required.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the </t>
+        </is>
+      </c>
+      <c r="D1289" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1290" s="17" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C1290" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Referral: NOT required.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: if the MBT is endoscopic, call the Erickson PA number on the ID car</t>
+        </is>
+      </c>
+      <c r="D1290" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: if the MBT is endoscopic, call the Erickson PA number on the ID card - Erickson requires PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1291" s="17" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="C1291" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either. The list names UHC Dual Complete as included.
+Referral: members must coordinate with their PCP; non-contracted providers need a referral form and PA (Dual Complete manual).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's </t>
+        </is>
+      </c>
+      <c r="D1291" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either. The list names UHC Dual Complete as included.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven. Medicaid wrap: experimental services are not AHCCCS b</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1292" s="17" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="C1292" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Referral: NOT required.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the </t>
+        </is>
+      </c>
+      <c r="D1292" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: first check the group # - if delegated to Optum or Banner, use the Optum tab. If the MBT is</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1293" s="17" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="C1293" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC Commercial list (eff. 9/1/2026). Arizona Pain Management Program: 64490-64495 need PA in all places of service; 64490/64493/64633/64635 need PA when done in hospital outpatient or ASC.
+Referral: REQUIRED - electronic PCP referral before the visit.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a p</t>
+        </is>
+      </c>
+      <c r="D1293" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC Commercial list (eff. 9/1/2026). Arizona Pain Management Program: 64490-64495 need PA in all places of service; 64490/64493/64633/64635 need PA when done in hospital outpatient or ASC.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1294" s="17" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="C1294" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC Commercial list (eff. 9/1/2026). Arizona Pain Management Program: 64490-64495 need PA in all places of service; 64490/64493/64633/64635 need PA when done in hospital outpatient or ASC.
+Referral: NOT required.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
+        </is>
+      </c>
+      <c r="D1294" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC Commercial list (eff. 9/1/2026). Arizona Pain Management Program: 64490-64495 need PA in all places of service; 64490/64493/64633/64635 need PA when done in hospital outpatient or ASC.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1295" s="17" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="C1295" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Individual Exchange list (eff. 9/1/2026). 64999 WOULD need PA. 64490, 64493, 64633, 64635 need PA + site-of-service review.
+Referral: REQUIRED in Arizona - UHC will not accept a PA without a referral on file. No out-of-network coverage.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination</t>
+        </is>
+      </c>
+      <c r="D1295" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Individual Exchange list (eff. 9/1/2026). 64999 WOULD need PA. 64490, 64493, 64633, 64635 need PA + site-of-service review.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1296" s="17" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C1296" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC Complete list (eff. 9/1/2026). 64999 WOULD need PA.
+Referral: REQUIRED - electronic PCP referral. No out-of-network coverage.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
+        </is>
+      </c>
+      <c r="D1296" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC Complete list (eff. 9/1/2026). 64999 WOULD need PA.
+Coverage: 2026T0107II - conventional (thermal) RFA covered with criteria and site-of-service review; endoscopic RFA/rhizotomy, pulsed, cooled, cryo, chemical and laser are UNPROVEN. 2026T0004WW: a positive diagnostic block = &gt;=50% relief.
+Action: if the MBT is endoscopic, expect a denial as unproven; get a predetermination before scheduling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1297" s="17" t="inlineStr">
+        <is>
+          <t>A39</t>
+        </is>
+      </c>
+      <c r="C1297" s="17" t="inlineStr">
+        <is>
+          <t>[ ] Referral on file where the plan requires one (UHC MA HMO/HMO-POS incl. D-SNP/C-SNP, Optum-delegated HMO - PCP submits it; UHC gated commercial; UHC AZ Exchange; Dual Complete).</t>
+        </is>
+      </c>
+      <c r="D1297" s="17" t="inlineStr">
+        <is>
+          <t>ROW REMOVED</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1298" s="17" t="inlineStr">
+        <is>
+          <t>D20</t>
+        </is>
+      </c>
+      <c r="C1298" s="17" t="inlineStr">
+        <is>
+          <t>Follows NCD 160.1 / L38801 (endoscopic evidence "insufficient"); commercial Ablative policy (endoscopic = unproven) may fill gaps. HMO/HMO-POS (incl. D-SNP/C-SNP HMO): PCP referral required.</t>
+        </is>
+      </c>
+      <c r="D1298" s="17" t="inlineStr">
+        <is>
+          <t>Follows NCD 160.1 / L38801 (endoscopic evidence "insufficient"); UHC commercial policy calls endoscopic rhizotomy unproven.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1299" s="17" t="inlineStr">
+        <is>
+          <t>D21</t>
+        </is>
+      </c>
+      <c r="C1299" s="17" t="inlineStr">
+        <is>
+          <t>HMO/HMO-POS: PCP referral to Optum required before the visit (except H5253-035, I-SNP, Erickson).</t>
+        </is>
+      </c>
+      <c r="D1299" s="17" t="inlineStr">
+        <is>
+          <t>Same coverage position as UHC MA (NCD 160.1 / L38801).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1300" s="17" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C1300" s="17" t="inlineStr">
+        <is>
+          <t>Referral on file</t>
+        </is>
+      </c>
+      <c r="D1300" s="17" t="inlineStr">
+        <is>
+          <t>Pre-service decision on optumproportal.com if endoscopic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1301" s="17" t="inlineStr">
+        <is>
+          <t>D22</t>
+        </is>
+      </c>
+      <c r="C1301" s="17" t="inlineStr">
+        <is>
+          <t>Endoscopic RFA/rhizotomy UNPROVEN. AZ Pain Management Program: 64490-64495 PA in all places of service. Gated plans need an electronic PCP referral; the AZ Exchange needs a PCP referral before any PA.</t>
+        </is>
+      </c>
+      <c r="D1301" s="17" t="inlineStr">
+        <is>
+          <t>Endoscopic RFA/rhizotomy UNPROVEN (2026T0107II). AZ Pain Management Program: 64490-64495 need PA in all places of service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1302" s="17" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C1302" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1302" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1303" s="17" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C1303" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1303" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1304" s="17" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C1304" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1304" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1305" s="17" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C1305" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1305" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1306" s="17" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C1306" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1306" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1307" s="17" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C1307" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1307" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1308" s="17" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="C1308" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1308" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1309" s="17" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="C1309" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1309" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1310" s="17" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="C1310" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1310" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1311" s="17" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="C1311" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1311" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1312" s="17" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="C1312" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1312" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1313" s="17" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="C1313" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1313" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1314" s="17" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C1314" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: confirm the referral is on file; if the MBT is endoscopic, request a pre-servi</t>
+        </is>
+      </c>
+      <c r="D1314" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Optum UHC MA list (Optum-direct providers) or the UHC MA list (all others).
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. Optum: new technology is not covered unless Optum approves it and PA is obtained.
+Action: if the MBT is endoscopic, request a pre-service decision on optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1315" s="17" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="C1315" s="17" t="inlineStr">
+        <is>
+          <t>Gated (referral required)</t>
+        </is>
+      </c>
+      <c r="D1315" s="17" t="inlineStr">
+        <is>
+          <t>Gated</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cite exact AMPM 820 sections and scope on the AHCCCS FFS row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiByUV3Zo1mhZNaeehe8GC
</commit_message>
<xml_diff>
--- a/Code Research/CPT_64772_Routing_2026.xlsx
+++ b/Code Research/CPT_64772_Routing_2026.xlsx
@@ -602,7 +602,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -652,7 +651,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
@@ -10017,7 +10015,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>AMPM 820 sections L.3.b, T and U; AMPM 810 (FFS UM)</t>
+          <t>AMPM 820 sec. L.3.b and L.5 (p.14); sec. T (p.21-22); sec. U (p.22)</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -10057,9 +10055,11 @@
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>PA: REQUIRED - elective outpatient surgery needs a surgeon PA AND a separate ASC/hospital PA (AMPM 820). Not needed if IHS/638 facility, emergency, or AHCCCS not primary.
+          <t>PA: REQUIRED. AMPM 820 L.3.b (p.14): "An Authorization is required ... for all FFS and DDD THP members: ... b. Elective and urgent outpatient surgical procedures". Sec. U (p.22): FFS surgeons "shall obtain a separate and distinct AHCCCS PA number from that of the facility PA number prior to providing elective/non-emergency surgeries". Sec. T: the ASC "shall obtain PA from AHCCCS DFSM for all outpatient surgeries".
+Applies ONLY to AHCCCS fee-for-service members (AIHP, Tribal ALTCS, TRBHA, DDD THP) - NOT to AHCCCS health plans (UHC Community Plan, Mercy Care, Health Choice, etc.).
+No PA needed (sec. III.1): emergency, AHCCCS not primary, IHS/638 provider or facility, retro eligibility. L.3.b refers to "section FF for exclusions", but the policy on file ends at section DD.
 Coverage: experimental services not covered (AMPM 320-B); moderate sedation by the performing physician not covered (Exh. 300-1).
-Action: submit both PAs on AHCCCS Online (fax 602-256-6591; phone 602-417-4400) before scheduling; put member name/DOB/ID on every page.</t>
+Action: submit surgeon PA and ASC PA to AHCCCS DFSM (AHCCCS Online; fax 602-256-6591; phone 602-417-4400) before scheduling.</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
@@ -11212,7 +11212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1315"/>
+  <dimension ref="A1:D1317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -40082,6 +40082,54 @@
         </is>
       </c>
     </row>
+    <row r="1316">
+      <c r="A1316" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS FFS</t>
+        </is>
+      </c>
+      <c r="B1316" s="17" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="C1316" s="17" t="inlineStr">
+        <is>
+          <t>AMPM 820 sections L.3.b, T and U; AMPM 810 (FFS UM)</t>
+        </is>
+      </c>
+      <c r="D1316" s="17" t="inlineStr">
+        <is>
+          <t>AMPM 820 sec. L.3.b and L.5 (p.14); sec. T (p.21-22); sec. U (p.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS FFS</t>
+        </is>
+      </c>
+      <c r="B1317" s="17" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C1317" s="17" t="inlineStr">
+        <is>
+          <t>PA: REQUIRED - elective outpatient surgery needs a surgeon PA AND a separate ASC/hospital PA (AMPM 820). Not needed if IHS/638 facility, emergency, or AHCCCS not primary.
+Coverage: experimental services not covered (AMPM 320-B); moderate sedation by the performing physician not covered (Exh. 300-1).
+Action: submit both PAs on AHCCCS Online (fax 602-256-6591; phone 602-417-4400) before scheduling; put member name/DOB/ID on every page.</t>
+        </is>
+      </c>
+      <c r="D1317" s="17" t="inlineStr">
+        <is>
+          <t>PA: REQUIRED. AMPM 820 L.3.b (p.14): "An Authorization is required ... for all FFS and DDD THP members: ... b. Elective and urgent outpatient surgical procedures". Sec. U (p.22): FFS surgeons "shall obtain a separate and distinct AHCCCS PA number from that of the facility PA number prior to providing elective/non-emergency surgeries". Sec. T: the ASC "shall obtain PA from AHCCCS DFSM for all outpatient surgeries".
+Applies ONLY to AHCCCS fee-for-service members (AIHP, Tribal ALTCS, TRBHA, DDD THP) - NOT to AHCCCS health plans (UHC Community Plan, Mercy Care, Health Choice, etc.).
+No PA needed (</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove phone and fax numbers; point every row to an online auth tool
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SiByUV3Zo1mhZNaeehe8GC
</commit_message>
<xml_diff>
--- a/Code Research/CPT_64772_Routing_2026.xlsx
+++ b/Code Research/CPT_64772_Routing_2026.xlsx
@@ -801,7 +801,7 @@
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>CALL (TPA / BCBS SC / home plan)</t>
+          <t>CHECK TPA / BCBS SC / home plan</t>
         </is>
       </c>
       <c r="D17" s="17" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>Call the TPA before scheduling</t>
+          <t>Check the TPA's auth tool before scheduling</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E18" s="17" t="inlineStr">
         <is>
-          <t>ACD 800-523-0023 / fax 800-266-3022</t>
+          <t>Request an ACD</t>
         </is>
       </c>
       <c r="F18" s="17" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>CALL BANNER</t>
+          <t>CHECK BANNER</t>
         </is>
       </c>
       <c r="D25" s="17" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>Ask Banner</t>
+          <t>Banner's auth tool</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
-          <t>AHCCCS Online / fax 602-256-6591</t>
+          <t>AHCCCS Online</t>
         </is>
       </c>
       <c r="F26" s="17" t="inlineStr">
@@ -1257,7 +1257,7 @@
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>- TPA groups (AHG, AmeriBen), BCBS SC, CHS, BlueCard home plans, Banner, delegated IPAs: call and record.</t>
+          <t>- TPA groups (AHG, AmeriBen), BCBS SC, CHS, BlueCard home plans, Banner, delegated IPAs: check each one's auth tool and record the result.</t>
         </is>
       </c>
     </row>
@@ -1587,17 +1587,17 @@
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>BCBS South Carolina (Blue Plan partner) - 800-868-1032</t>
+          <t>BCBS South Carolina (Blue Plan partner)</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>CALL BCBS SC</t>
+          <t>CHECK BCBS SC</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>No online tool on file - call BCBS South Carolina 800-868-1032</t>
+          <t>BCBS South Carolina's auth tool (not on file)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -1617,12 +1617,12 @@
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
@@ -1649,7 +1649,7 @@
         <is>
           <t>PA: decided by BCBS South Carolina (AZ Blue code-list Introduction). No BCBS SC list on file.
 Note: IVR also appears in the Standard list prefix header.
-Action: call BCBS SC 800-868-1032 before scheduling; record name, date and reference #.</t>
+Action: check BCBS SC's auth tool before scheduling; record the result.</t>
         </is>
       </c>
       <c r="U3" s="3" t="inlineStr">
@@ -1689,17 +1689,17 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>American Health Group (AHG) - PA and medical policy, 800-847-7605</t>
+          <t>American Health Group (AHG) - PA and medical policy</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>CALL AHG</t>
+          <t>CHECK AHG</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>No online tool on file - call American Health Group 800-847-7605</t>
+          <t>American Health Group's auth tool (not on file)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="O4" s="7" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
@@ -1749,8 +1749,8 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>PA: decided by American Health Group; the group may customize PA (AZ Blue TPA document, 07/2026). No AHG list on file.
-Action: call AHG 800-847-7605 before scheduling; record reference #. Claims still go to AZ Blue (EDI 53589).</t>
+          <t>PA: decided by American Health Group; the group may customize PA (AZ Blue and TPA Jointly Administered Plans, as of 07/2026). No AHG list on file.
+Action: check AHG's auth tool before scheduling; record the result. Claims still go to AZ Blue (EDI 53589).</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
@@ -1795,12 +1795,12 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>CALL AMERIBEN</t>
+          <t>CHECK AMERIBEN</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>AmeriBen PA line by group: JCG 855-240-3698; JKS 855-961-5401; JPZ 855-778-9053; K8Y/K8Z 800-388-3193; MKQ 866-947-9522; PTP 833-359-2505</t>
+          <t>AmeriBen's auth tool for the group (not on file)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -1820,12 +1820,12 @@
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
@@ -1850,8 +1850,8 @@
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>PA: decided by AmeriBen; the group may customize PA (AZ Blue TPA document, 07/2026). No AmeriBen list on file.
-Action: call the AmeriBen line for the prefix (column J) before scheduling; record reference #. Claims go to AZ Blue (EDI 53589).</t>
+          <t>PA: decided by AmeriBen; the group may customize PA (AZ Blue and TPA Jointly Administered Plans, as of 07/2026). No AmeriBen list on file.
+Action: check AmeriBen's auth tool before scheduling; record the result. Claims go to AZ Blue (EDI 53589).</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -1892,12 +1892,12 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>CALL TPA</t>
+          <t>CHECK TPA</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Call the number on the ID card</t>
+          <t>The TPA's auth tool (TPA named on the ID card)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -1917,12 +1917,12 @@
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -1948,7 +1948,7 @@
       <c r="T6" s="3" t="inlineStr">
         <is>
           <t>PA: decided by the TPA on the ID card (AZ Blue code-list Introduction). No list on file.
-Action: call the number on the ID card before scheduling; record reference #.</t>
+Action: check the TPA's auth tool before scheduling; record the result.</t>
         </is>
       </c>
       <c r="U6" s="3" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>CALL HOME PLAN</t>
+          <t>CHECK HOME PLAN</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -3799,7 +3799,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -5720,12 +5720,12 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>CALL PLAN ON CARD</t>
+          <t>CHECK PLAN ON CARD</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Care-management delegation does not carry prior-auth authority. Check with the plan on the card.</t>
+          <t>Use the auth tool of the plan on the ID card</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -5825,12 +5825,12 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>CALL IPA</t>
+          <t>CHECK IPA</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>Each IPA runs its own UM with its own criteria - ask each one separately</t>
+          <t>The IPA's own auth tool (not on file)</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -5850,12 +5850,12 @@
       </c>
       <c r="N23" s="3" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="P23" s="3" t="inlineStr">
@@ -5881,7 +5881,7 @@
       <c r="T23" s="3" t="inlineStr">
         <is>
           <t>PA: the delegated IPA's own rules apply (UHC MA PA list: providers contracted with a delegated IPA must follow its protocols). No IPA list on file.
-Action: call the IPA before scheduling; record reference #.</t>
+Action: check the IPA's auth tool before scheduling; record the result.</t>
         </is>
       </c>
       <c r="U23" s="3" t="inlineStr">
@@ -5938,12 +5938,12 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>CALL BANNER</t>
+          <t>CHECK BANNER</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Per the Banner AZ QRG - NOT optumproportal.com</t>
+          <t>Banner's auth tool (not on file) - not optumproportal.com</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -5963,12 +5963,12 @@
       </c>
       <c r="N24" s="3" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="O24" s="7" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="P24" s="3" t="inlineStr">
@@ -5994,7 +5994,7 @@
       <c r="T24" s="3" t="inlineStr">
         <is>
           <t>PA: these group numbers are delegated to Banner (UHC MA PA list, eff. 9/1/2026). Banner's list is not on file.
-Action: call Banner (number on the ID card) before scheduling; do not use optumproportal.com.</t>
+Action: check Banner's auth tool before scheduling; do not use optumproportal.com.</t>
         </is>
       </c>
       <c r="U24" s="3" t="inlineStr">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>Ask the Optum provider rep which plan carries group 96001</t>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -6302,7 +6302,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -6498,7 +6498,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -6596,7 +6596,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -6792,7 +6792,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Erickson MSR / prior authorization number on the back of the ID card; UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+          <t>Erickson prior authorization contact on the back of the ID card; UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -6844,7 +6844,7 @@
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
-Action: if the MBT is endoscopic, call the Erickson PA number on the ID card - Erickson requires PA for experimental/investigational services.</t>
+Action: if the MBT is endoscopic, request PA through the Erickson contact on the ID card - Erickson requires PA for experimental/investigational services.</t>
         </is>
       </c>
       <c r="U7" s="3" t="inlineStr">
@@ -6890,7 +6890,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 1-800-445-1638</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -6942,7 +6942,7 @@
         <is>
           <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either. The list names UHC Dual Complete as included.
 Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven. Medicaid wrap: experimental services are not AHCCCS benefits.
-Action: PA line 800-445-1638 if needed. QMB members owe $0 - do not bill the member.</t>
+Action: QMB members owe $0 - do not bill the member.</t>
         </is>
       </c>
       <c r="U8" s="3" t="inlineStr">
@@ -6988,7 +6988,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -7388,7 +7388,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 800-445-1638</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -7440,7 +7440,7 @@
         <is>
           <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
 Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
-Action: if the MBT is endoscopic, expect denial as experimental. PA line 800-445-1638.</t>
+Action: if the MBT is endoscopic, expect denial as experimental.</t>
         </is>
       </c>
       <c r="U13" s="3" t="inlineStr">
@@ -7481,12 +7481,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>CALL TPA</t>
+          <t>CHECK TPA</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Per that supplement. UMR: umr.com</t>
+          <t>The TPA's auth tool per the ID card (UMR: umr.com)</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -7506,12 +7506,12 @@
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
-          <t>No list on file - call (see T)</t>
+          <t>No list on file - see T</t>
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr">
@@ -7537,7 +7537,7 @@
       <c r="T14" s="3" t="inlineStr">
         <is>
           <t>PA: set by each group's plan document and TPA supplement - no list on file.
-Action: check the member's ID card / portal (UMR: umr.com) and call before scheduling; record reference #.</t>
+Action: check the TPA's auth tool (UMR: umr.com) before scheduling; record the result.</t>
         </is>
       </c>
       <c r="U14" s="3" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 800-445-1638</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -8053,7 +8053,7 @@
         <is>
           <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
 Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
-Action: if the MBT is endoscopic, expect denial as experimental. PA line 800-445-1638.</t>
+Action: if the MBT is endoscopic, expect denial as experimental.</t>
         </is>
       </c>
       <c r="U19" s="3" t="inlineStr">
@@ -8099,7 +8099,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -8151,7 +8151,7 @@
         <is>
           <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
 Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
-Action: if the MBT is endoscopic, expect denial as experimental. PA line 877-842-3210.</t>
+Action: if the MBT is endoscopic, expect denial as experimental.</t>
         </is>
       </c>
       <c r="U20" s="3" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Availity auth tool and Cohere Health auth tool - both checked: not required (your check). ACD: 800-523-0023 / fax 800-266-3022</t>
+          <t>Availity auth tool and Cohere Health auth tool - both checked: not required (your check)</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -8775,7 +8775,7 @@
         <is>
           <t>PA: NOT required - 64772 is not on the Humana MA/D-SNP list (eff. 7/1/2026, rev. 9/1/2026); Availity and Cohere returned not required (your check). 64999 and facet codes 64490-64495, 64633-64636 DO need PA through Cohere.
 Coverage: HUM-1168-008 - endoscopic RF ablation/rhizotomy for any indication, including the facet nerve, is NOT reasonable and necessary. Conventional facet RFA follows L38801/A58403.
-Action: request an Advance Coverage Determination before scheduling (800-523-0023 / fax 800-266-3022 / PO Box 14601, Lexington KY 40512-4601). Without it, a post-payment denial is likely and the member cannot be billed.</t>
+Action: request an Advance Coverage Determination before scheduling. Without it, a post-payment denial is likely and the member cannot be billed.</t>
         </is>
       </c>
       <c r="U2" s="10" t="inlineStr">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>AHCCCS Online provider portal; Medical PA fax 602-256-6591; phone 602-417-4400 / 800-433-0425</t>
+          <t>AHCCCS Online provider portal</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -10057,7 +10057,7 @@
 Applies ONLY to AHCCCS fee-for-service members (AIHP, Tribal ALTCS, TRBHA, DDD THP) - NOT to AHCCCS health plans (UHC Community Plan, Mercy Care, Health Choice, etc.).
 No PA needed (sec. III.1): emergency, AHCCCS not primary, IHS/638 provider or facility, retro eligibility. L.3.b refers to "section FF for exclusions", but the policy on file ends at section DD.
 Coverage: experimental services not covered (AMPM 320-B); moderate sedation by the performing physician not covered (Exh. 300-1).
-Action: submit surgeon PA and ASC PA to AHCCCS DFSM (AHCCCS Online; fax 602-256-6591; phone 602-417-4400) before scheduling.</t>
+Action: submit surgeon PA and ASC PA to AHCCCS DFSM on AHCCCS Online before scheduling.</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
@@ -11210,7 +11210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1541"/>
+  <dimension ref="A1:D1630"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -45039,6 +45039,1969 @@
         </is>
       </c>
     </row>
+    <row r="1543">
+      <c r="A1543" s="15" t="inlineStr">
+        <is>
+          <t>Round 8 - phone and fax numbers removed (auths are checked in online tools)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1544" s="17" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="C1544" s="17" t="inlineStr">
+        <is>
+          <t>BCBS South Carolina (Blue Plan partner) - 800-868-1032</t>
+        </is>
+      </c>
+      <c r="D1544" s="17" t="inlineStr">
+        <is>
+          <t>BCBS South Carolina (Blue Plan partner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1545" s="17" t="inlineStr">
+        <is>
+          <t>I3</t>
+        </is>
+      </c>
+      <c r="C1545" s="17" t="inlineStr">
+        <is>
+          <t>CALL BCBS SC</t>
+        </is>
+      </c>
+      <c r="D1545" s="17" t="inlineStr">
+        <is>
+          <t>CHECK BCBS SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1546" s="17" t="inlineStr">
+        <is>
+          <t>J3</t>
+        </is>
+      </c>
+      <c r="C1546" s="17" t="inlineStr">
+        <is>
+          <t>No online tool on file - call BCBS South Carolina 800-868-1032</t>
+        </is>
+      </c>
+      <c r="D1546" s="17" t="inlineStr">
+        <is>
+          <t>BCBS South Carolina's auth tool (not on file)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1547" s="17" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C1547" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by BCBS South Carolina (AZ Blue code-list Introduction). No BCBS SC list on file.
+Note: IVR also appears in the Standard list prefix header.
+Action: call BCBS SC 800-868-1032 before scheduling; record name, date and reference #.</t>
+        </is>
+      </c>
+      <c r="D1547" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by BCBS South Carolina (AZ Blue code-list Introduction). No BCBS SC list on file.
+Note: IVR also appears in the Standard list prefix header.
+Action: check BCBS SC's auth tool before scheduling; record the result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1548" s="17" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="C1548" s="17" t="inlineStr">
+        <is>
+          <t>American Health Group (AHG) - PA and medical policy, 800-847-7605</t>
+        </is>
+      </c>
+      <c r="D1548" s="17" t="inlineStr">
+        <is>
+          <t>American Health Group (AHG) - PA and medical policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1549" s="17" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="C1549" s="17" t="inlineStr">
+        <is>
+          <t>CALL AHG</t>
+        </is>
+      </c>
+      <c r="D1549" s="17" t="inlineStr">
+        <is>
+          <t>CHECK AHG</t>
+        </is>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1550" s="17" t="inlineStr">
+        <is>
+          <t>J4</t>
+        </is>
+      </c>
+      <c r="C1550" s="17" t="inlineStr">
+        <is>
+          <t>No online tool on file - call American Health Group 800-847-7605</t>
+        </is>
+      </c>
+      <c r="D1550" s="17" t="inlineStr">
+        <is>
+          <t>American Health Group's auth tool (not on file)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1551" s="17" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C1551" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by American Health Group; the group may customize PA (AZ Blue TPA document, 07/2026). No AHG list on file.
+Action: call AHG 800-847-7605 before scheduling; record reference #. Claims still go to AZ Blue (EDI 53589).</t>
+        </is>
+      </c>
+      <c r="D1551" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by American Health Group; the group may customize PA (AZ Blue and TPA Jointly Administered Plans, as of 07/2026). No AHG list on file.
+Action: check AHG's auth tool before scheduling; record the result. Claims still go to AZ Blue (EDI 53589).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1552" s="17" t="inlineStr">
+        <is>
+          <t>I5</t>
+        </is>
+      </c>
+      <c r="C1552" s="17" t="inlineStr">
+        <is>
+          <t>CALL AMERIBEN</t>
+        </is>
+      </c>
+      <c r="D1552" s="17" t="inlineStr">
+        <is>
+          <t>CHECK AMERIBEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1553" s="17" t="inlineStr">
+        <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="C1553" s="17" t="inlineStr">
+        <is>
+          <t>AmeriBen PA line by group: JCG 855-240-3698; JKS 855-961-5401; JPZ 855-778-9053; K8Y/K8Z 800-388-3193; MKQ 866-947-9522; PTP 833-359-2505</t>
+        </is>
+      </c>
+      <c r="D1553" s="17" t="inlineStr">
+        <is>
+          <t>AmeriBen's auth tool for the group (not on file)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1554" s="17" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="C1554" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by AmeriBen; the group may customize PA (AZ Blue TPA document, 07/2026). No AmeriBen list on file.
+Action: call the AmeriBen line for the prefix (column J) before scheduling; record reference #. Claims go to AZ Blue (EDI 53589).</t>
+        </is>
+      </c>
+      <c r="D1554" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by AmeriBen; the group may customize PA (AZ Blue and TPA Jointly Administered Plans, as of 07/2026). No AmeriBen list on file.
+Action: check AmeriBen's auth tool before scheduling; record the result. Claims go to AZ Blue (EDI 53589).</t>
+        </is>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1555" s="17" t="inlineStr">
+        <is>
+          <t>I6</t>
+        </is>
+      </c>
+      <c r="C1555" s="17" t="inlineStr">
+        <is>
+          <t>CALL TPA</t>
+        </is>
+      </c>
+      <c r="D1555" s="17" t="inlineStr">
+        <is>
+          <t>CHECK TPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1556" s="17" t="inlineStr">
+        <is>
+          <t>J6</t>
+        </is>
+      </c>
+      <c r="C1556" s="17" t="inlineStr">
+        <is>
+          <t>Call the number on the ID card</t>
+        </is>
+      </c>
+      <c r="D1556" s="17" t="inlineStr">
+        <is>
+          <t>The TPA's auth tool (TPA named on the ID card)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1557" s="17" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="C1557" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by the TPA on the ID card (AZ Blue code-list Introduction). No list on file.
+Action: call the number on the ID card before scheduling; record reference #.</t>
+        </is>
+      </c>
+      <c r="D1557" s="17" t="inlineStr">
+        <is>
+          <t>PA: decided by the TPA on the ID card (AZ Blue code-list Introduction). No list on file.
+Action: check the TPA's auth tool before scheduling; record the result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1558" s="17" t="inlineStr">
+        <is>
+          <t>I17</t>
+        </is>
+      </c>
+      <c r="C1558" s="17" t="inlineStr">
+        <is>
+          <t>CALL HOME PLAN</t>
+        </is>
+      </c>
+      <c r="D1558" s="17" t="inlineStr">
+        <is>
+          <t>CHECK HOME PLAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1559" s="17" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="C1559" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1559" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1560" s="17" t="inlineStr">
+        <is>
+          <t>O3</t>
+        </is>
+      </c>
+      <c r="C1560" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1560" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1561" s="17" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="C1561" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1561" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1562" s="17" t="inlineStr">
+        <is>
+          <t>O4</t>
+        </is>
+      </c>
+      <c r="C1562" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1562" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1563" s="17" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="C1563" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1563" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1564" s="17" t="inlineStr">
+        <is>
+          <t>O5</t>
+        </is>
+      </c>
+      <c r="C1564" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1564" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1565" s="17" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="C1565" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1565" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1566" s="17" t="inlineStr">
+        <is>
+          <t>O6</t>
+        </is>
+      </c>
+      <c r="C1566" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1566" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1567" s="17" t="inlineStr">
+        <is>
+          <t>J8</t>
+        </is>
+      </c>
+      <c r="C1567" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+      <c r="D1567" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1568" s="17" t="inlineStr">
+        <is>
+          <t>J10</t>
+        </is>
+      </c>
+      <c r="C1568" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+      <c r="D1568" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" s="17" t="inlineStr">
+        <is>
+          <t>BCBS</t>
+        </is>
+      </c>
+      <c r="B1569" s="17" t="inlineStr">
+        <is>
+          <t>J11</t>
+        </is>
+      </c>
+      <c r="C1569" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+      <c r="D1569" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1570" s="17" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="C1570" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1570" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1571" s="17" t="inlineStr">
+        <is>
+          <t>J3</t>
+        </is>
+      </c>
+      <c r="C1571" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1571" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1572" s="17" t="inlineStr">
+        <is>
+          <t>J4</t>
+        </is>
+      </c>
+      <c r="C1572" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1572" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1573" s="17" t="inlineStr">
+        <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="C1573" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1573" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1574" s="17" t="inlineStr">
+        <is>
+          <t>J6</t>
+        </is>
+      </c>
+      <c r="C1574" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1574" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1575" s="17" t="inlineStr">
+        <is>
+          <t>J7</t>
+        </is>
+      </c>
+      <c r="C1575" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1575" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1576" s="17" t="inlineStr">
+        <is>
+          <t>J8</t>
+        </is>
+      </c>
+      <c r="C1576" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1576" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1577" s="17" t="inlineStr">
+        <is>
+          <t>J9</t>
+        </is>
+      </c>
+      <c r="C1577" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1577" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1578" s="17" t="inlineStr">
+        <is>
+          <t>J10</t>
+        </is>
+      </c>
+      <c r="C1578" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1578" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1579" s="17" t="inlineStr">
+        <is>
+          <t>J11</t>
+        </is>
+      </c>
+      <c r="C1579" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1579" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1580" s="17" t="inlineStr">
+        <is>
+          <t>J12</t>
+        </is>
+      </c>
+      <c r="C1580" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1580" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1581" s="17" t="inlineStr">
+        <is>
+          <t>J13</t>
+        </is>
+      </c>
+      <c r="C1581" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1581" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1582" s="17" t="inlineStr">
+        <is>
+          <t>J14</t>
+        </is>
+      </c>
+      <c r="C1582" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1582" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1583" s="17" t="inlineStr">
+        <is>
+          <t>J15</t>
+        </is>
+      </c>
+      <c r="C1583" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+      <c r="D1583" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1584" s="17" t="inlineStr">
+        <is>
+          <t>J16</t>
+        </is>
+      </c>
+      <c r="C1584" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com; phone 877-370-2845 if portal down. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+      <c r="D1584" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com. If not Optum-direct: Availity auth tool (prior auth workflow); AZ Blue PA lookup tool: azblue.com/lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1585" s="17" t="inlineStr">
+        <is>
+          <t>I22</t>
+        </is>
+      </c>
+      <c r="C1585" s="17" t="inlineStr">
+        <is>
+          <t>CALL PLAN ON CARD</t>
+        </is>
+      </c>
+      <c r="D1585" s="17" t="inlineStr">
+        <is>
+          <t>CHECK PLAN ON CARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1586" s="17" t="inlineStr">
+        <is>
+          <t>I23</t>
+        </is>
+      </c>
+      <c r="C1586" s="17" t="inlineStr">
+        <is>
+          <t>CALL IPA</t>
+        </is>
+      </c>
+      <c r="D1586" s="17" t="inlineStr">
+        <is>
+          <t>CHECK IPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1587" s="17" t="inlineStr">
+        <is>
+          <t>I24</t>
+        </is>
+      </c>
+      <c r="C1587" s="17" t="inlineStr">
+        <is>
+          <t>CALL BANNER</t>
+        </is>
+      </c>
+      <c r="D1587" s="17" t="inlineStr">
+        <is>
+          <t>CHECK BANNER</t>
+        </is>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1588" s="17" t="inlineStr">
+        <is>
+          <t>J22</t>
+        </is>
+      </c>
+      <c r="C1588" s="17" t="inlineStr">
+        <is>
+          <t>Care-management delegation does not carry prior-auth authority. Check with the plan on the card.</t>
+        </is>
+      </c>
+      <c r="D1588" s="17" t="inlineStr">
+        <is>
+          <t>Use the auth tool of the plan on the ID card</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1589" s="17" t="inlineStr">
+        <is>
+          <t>J23</t>
+        </is>
+      </c>
+      <c r="C1589" s="17" t="inlineStr">
+        <is>
+          <t>Each IPA runs its own UM with its own criteria - ask each one separately</t>
+        </is>
+      </c>
+      <c r="D1589" s="17" t="inlineStr">
+        <is>
+          <t>The IPA's own auth tool (not on file)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1590" s="17" t="inlineStr">
+        <is>
+          <t>J24</t>
+        </is>
+      </c>
+      <c r="C1590" s="17" t="inlineStr">
+        <is>
+          <t>Per the Banner AZ QRG - NOT optumproportal.com</t>
+        </is>
+      </c>
+      <c r="D1590" s="17" t="inlineStr">
+        <is>
+          <t>Banner's auth tool (not on file) - not optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1591" s="17" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="C1591" s="17" t="inlineStr">
+        <is>
+          <t>PA: the delegated IPA's own rules apply (UHC MA PA list: providers contracted with a delegated IPA must follow its protocols). No IPA list on file.
+Action: call the IPA before scheduling; record reference #.</t>
+        </is>
+      </c>
+      <c r="D1591" s="17" t="inlineStr">
+        <is>
+          <t>PA: the delegated IPA's own rules apply (UHC MA PA list: providers contracted with a delegated IPA must follow its protocols). No IPA list on file.
+Action: check the IPA's auth tool before scheduling; record the result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1592" s="17" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="C1592" s="17" t="inlineStr">
+        <is>
+          <t>PA: these group numbers are delegated to Banner (UHC MA PA list, eff. 9/1/2026). Banner's list is not on file.
+Action: call Banner (number on the ID card) before scheduling; do not use optumproportal.com.</t>
+        </is>
+      </c>
+      <c r="D1592" s="17" t="inlineStr">
+        <is>
+          <t>PA: these group numbers are delegated to Banner (UHC MA PA list, eff. 9/1/2026). Banner's list is not on file.
+Action: check Banner's auth tool before scheduling; do not use optumproportal.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1593" s="17" t="inlineStr">
+        <is>
+          <t>J25</t>
+        </is>
+      </c>
+      <c r="C1593" s="17" t="inlineStr">
+        <is>
+          <t>Ask the Optum provider rep which plan carries group 96001</t>
+        </is>
+      </c>
+      <c r="D1593" s="17" t="inlineStr">
+        <is>
+          <t>Curo (Optum auth tool) via Optum Pro portal: optumproportal.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1594" s="17" t="inlineStr">
+        <is>
+          <t>N23</t>
+        </is>
+      </c>
+      <c r="C1594" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1594" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1595" s="17" t="inlineStr">
+        <is>
+          <t>O23</t>
+        </is>
+      </c>
+      <c r="C1595" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1595" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1596" s="17" t="inlineStr">
+        <is>
+          <t>N24</t>
+        </is>
+      </c>
+      <c r="C1596" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1596" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" s="17" t="inlineStr">
+        <is>
+          <t>Optum</t>
+        </is>
+      </c>
+      <c r="B1597" s="17" t="inlineStr">
+        <is>
+          <t>O24</t>
+        </is>
+      </c>
+      <c r="C1597" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1597" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1598" s="17" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="C1598" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1598" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1599" s="17" t="inlineStr">
+        <is>
+          <t>J3</t>
+        </is>
+      </c>
+      <c r="C1599" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1599" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1600" s="17" t="inlineStr">
+        <is>
+          <t>J4</t>
+        </is>
+      </c>
+      <c r="C1600" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1600" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1601" s="17" t="inlineStr">
+        <is>
+          <t>J5</t>
+        </is>
+      </c>
+      <c r="C1601" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1601" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1602" s="17" t="inlineStr">
+        <is>
+          <t>J6</t>
+        </is>
+      </c>
+      <c r="C1602" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1602" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1603" s="17" t="inlineStr">
+        <is>
+          <t>J8</t>
+        </is>
+      </c>
+      <c r="C1603" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 1-800-445-1638</t>
+        </is>
+      </c>
+      <c r="D1603" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1604" s="17" t="inlineStr">
+        <is>
+          <t>J9</t>
+        </is>
+      </c>
+      <c r="C1604" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1604" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1605" s="17" t="inlineStr">
+        <is>
+          <t>J13</t>
+        </is>
+      </c>
+      <c r="C1605" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 800-445-1638</t>
+        </is>
+      </c>
+      <c r="D1605" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1606" s="17" t="inlineStr">
+        <is>
+          <t>J18</t>
+        </is>
+      </c>
+      <c r="C1606" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1606" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1607" s="17" t="inlineStr">
+        <is>
+          <t>J19</t>
+        </is>
+      </c>
+      <c r="C1607" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 800-445-1638</t>
+        </is>
+      </c>
+      <c r="D1607" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1608" s="17" t="inlineStr">
+        <is>
+          <t>J20</t>
+        </is>
+      </c>
+      <c r="C1608" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan); phone 877-842-3210</t>
+        </is>
+      </c>
+      <c r="D1608" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1609" s="17" t="inlineStr">
+        <is>
+          <t>J7</t>
+        </is>
+      </c>
+      <c r="C1609" s="17" t="inlineStr">
+        <is>
+          <t>Erickson MSR / prior authorization number on the back of the ID card; UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+      <c r="D1609" s="17" t="inlineStr">
+        <is>
+          <t>Erickson prior authorization contact on the back of the ID card; UnitedHealthcare Provider Portal &gt; Prior Authorization and Notification tool (UHCprovider.com/paan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1610" s="17" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="C1610" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: if the MBT is endoscopic, call the Erickson PA number on the ID card - Erickson requires PA</t>
+        </is>
+      </c>
+      <c r="D1610" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven.
+Action: if the MBT is endoscopic, request PA through the Erickson contact on the ID card - Erickson</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1611" s="17" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="C1611" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either. The list names UHC Dual Complete as included.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven. Medicaid wrap: experimental services are not AHCCCS b</t>
+        </is>
+      </c>
+      <c r="D1611" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the UHC MA PA list (eff. 9/1/2026); no facet codes are on it either. The list names UHC Dual Complete as included.
+Coverage: NCD 160.1 allows nerve cutting case by case. L38801 criteria for facet denervation: 2 diagnostic MBBs, each &gt;=80% relief, &gt;=2 weeks apart; &gt;=3 months pain; failed conservative care; max 2 sessions per region per 12 months. L38801 states there is insufficient evidence for ENDOSCOPIC dorsal ramus rhizotomy. UHC's commercial policy 2026T0107II lists endoscopic RFA/rhizotomy as unproven. Medicaid wrap: experimental services are not AHCCCS b</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1612" s="17" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="C1612" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
+Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
+Action: if the MBT is endoscopic, expect denial as experimental. PA line 800-445-1638.</t>
+        </is>
+      </c>
+      <c r="D1612" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
+Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
+Action: if the MBT is endoscopic, expect denial as experimental.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1613" s="17" t="inlineStr">
+        <is>
+          <t>T19</t>
+        </is>
+      </c>
+      <c r="C1613" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
+Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
+Action: if the MBT is endoscopic, expect denial as experimental. PA line 800-445-1638.</t>
+        </is>
+      </c>
+      <c r="D1613" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
+Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
+Action: if the MBT is endoscopic, expect denial as experimental.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1614" s="17" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="C1614" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
+Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
+Action: if the MBT is endoscopic, expect denial as experimental. PA line 877-842-3210.</t>
+        </is>
+      </c>
+      <c r="D1614" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the list (eff. 9/1/2026). 64490 and 64493 need PA. Anything experimental/investigational needs PA and is not a covered AHCCCS benefit.
+Coverage: CS001.T - endoscopic RFA/rhizotomy is unproven. Moderate sedation by the performing physician is not covered (AMPM Exh. 300-1). Provider must be AHCCCS-registered.
+Action: if the MBT is endoscopic, expect denial as experimental.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1615" s="17" t="inlineStr">
+        <is>
+          <t>I14</t>
+        </is>
+      </c>
+      <c r="C1615" s="17" t="inlineStr">
+        <is>
+          <t>CALL TPA</t>
+        </is>
+      </c>
+      <c r="D1615" s="17" t="inlineStr">
+        <is>
+          <t>CHECK TPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1616" s="17" t="inlineStr">
+        <is>
+          <t>J14</t>
+        </is>
+      </c>
+      <c r="C1616" s="17" t="inlineStr">
+        <is>
+          <t>Per that supplement. UMR: umr.com</t>
+        </is>
+      </c>
+      <c r="D1616" s="17" t="inlineStr">
+        <is>
+          <t>The TPA's auth tool per the ID card (UMR: umr.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1617" s="17" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C1617" s="17" t="inlineStr">
+        <is>
+          <t>PA: set by each group's plan document and TPA supplement - no list on file.
+Action: check the member's ID card / portal (UMR: umr.com) and call before scheduling; record reference #.</t>
+        </is>
+      </c>
+      <c r="D1617" s="17" t="inlineStr">
+        <is>
+          <t>PA: set by each group's plan document and TPA supplement - no list on file.
+Action: check the TPA's auth tool (UMR: umr.com) before scheduling; record the result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1618" s="17" t="inlineStr">
+        <is>
+          <t>N14</t>
+        </is>
+      </c>
+      <c r="C1618" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1618" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" s="17" t="inlineStr">
+        <is>
+          <t>UnitedHealthcare</t>
+        </is>
+      </c>
+      <c r="B1619" s="17" t="inlineStr">
+        <is>
+          <t>O14</t>
+        </is>
+      </c>
+      <c r="C1619" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - call (see T)</t>
+        </is>
+      </c>
+      <c r="D1619" s="17" t="inlineStr">
+        <is>
+          <t>No list on file - see T</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B1620" s="17" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="C1620" s="17" t="inlineStr">
+        <is>
+          <t>Availity auth tool and Cohere Health auth tool - both checked: not required (your check). ACD: 800-523-0023 / fax 800-266-3022</t>
+        </is>
+      </c>
+      <c r="D1620" s="17" t="inlineStr">
+        <is>
+          <t>Availity auth tool and Cohere Health auth tool - both checked: not required (your check)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" s="17" t="inlineStr">
+        <is>
+          <t>Humana</t>
+        </is>
+      </c>
+      <c r="B1621" s="17" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C1621" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Humana MA/D-SNP list (eff. 7/1/2026, rev. 9/1/2026); Availity and Cohere returned not required (your check). 64999 and facet codes 64490-64495, 64633-64636 DO need PA through Cohere.
+Coverage: HUM-1168-008 - endoscopic RF ablation/rhizotomy for any indication, including the facet nerve, is NOT reasonable and necessary. Conventional facet RFA follows L38801/A58403.
+Action: request an Advance Coverage Determination before scheduling (800-523-0023 / fax 800-266-3022 / PO Box 14601, Lexington KY 40512-4601). Without it, a post-payment denial is likely and the</t>
+        </is>
+      </c>
+      <c r="D1621" s="17" t="inlineStr">
+        <is>
+          <t>PA: NOT required - 64772 is not on the Humana MA/D-SNP list (eff. 7/1/2026, rev. 9/1/2026); Availity and Cohere returned not required (your check). 64999 and facet codes 64490-64495, 64633-64636 DO need PA through Cohere.
+Coverage: HUM-1168-008 - endoscopic RF ablation/rhizotomy for any indication, including the facet nerve, is NOT reasonable and necessary. Conventional facet RFA follows L38801/A58403.
+Action: request an Advance Coverage Determination before scheduling. Without it, a post-payment denial is likely and the member cannot be billed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS FFS</t>
+        </is>
+      </c>
+      <c r="B1622" s="17" t="inlineStr">
+        <is>
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="C1622" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS Online provider portal; Medical PA fax 602-256-6591; phone 602-417-4400 / 800-433-0425</t>
+        </is>
+      </c>
+      <c r="D1622" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS Online provider portal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS FFS</t>
+        </is>
+      </c>
+      <c r="B1623" s="17" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C1623" s="17" t="inlineStr">
+        <is>
+          <t>PA: REQUIRED. AMPM 820 L.3.b (p.14): "An Authorization is required ... for all FFS and DDD THP members: ... b. Elective and urgent outpatient surgical procedures". Sec. U (p.22): FFS surgeons "shall obtain a separate and distinct AHCCCS PA number from that of the facility PA number prior to providing elective/non-emergency surgeries". Sec. T: the ASC "shall obtain PA from AHCCCS DFSM for all outpatient surgeries".
+Applies ONLY to AHCCCS fee-for-service members (AIHP, Tribal ALTCS, TRBHA, DDD THP) - NOT to AHCCCS health plans (UHC Community Plan, Mercy Care, Health Choice, etc.).
+No PA needed (</t>
+        </is>
+      </c>
+      <c r="D1623" s="17" t="inlineStr">
+        <is>
+          <t>PA: REQUIRED. AMPM 820 L.3.b (p.14): "An Authorization is required ... for all FFS and DDD THP members: ... b. Elective and urgent outpatient surgical procedures". Sec. U (p.22): FFS surgeons "shall obtain a separate and distinct AHCCCS PA number from that of the facility PA number prior to providing elective/non-emergency surgeries". Sec. T: the ASC "shall obtain PA from AHCCCS DFSM for all outpatient surgeries".
+Applies ONLY to AHCCCS fee-for-service members (AIHP, Tribal ALTCS, TRBHA, DDD THP) - NOT to AHCCCS health plans (UHC Community Plan, Mercy Care, Health Choice, etc.).
+No PA needed (</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1624" s="17" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="C1624" s="17" t="inlineStr">
+        <is>
+          <t>CALL (TPA / BCBS SC / home plan)</t>
+        </is>
+      </c>
+      <c r="D1624" s="17" t="inlineStr">
+        <is>
+          <t>CHECK TPA / BCBS SC / home plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1625" s="17" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C1625" s="17" t="inlineStr">
+        <is>
+          <t>Call the TPA before scheduling</t>
+        </is>
+      </c>
+      <c r="D1625" s="17" t="inlineStr">
+        <is>
+          <t>Check the TPA's auth tool before scheduling</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1626" s="17" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C1626" s="17" t="inlineStr">
+        <is>
+          <t>ACD 800-523-0023 / fax 800-266-3022</t>
+        </is>
+      </c>
+      <c r="D1626" s="17" t="inlineStr">
+        <is>
+          <t>Request an ACD</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1627" s="17" t="inlineStr">
+        <is>
+          <t>C25</t>
+        </is>
+      </c>
+      <c r="C1627" s="17" t="inlineStr">
+        <is>
+          <t>CALL BANNER</t>
+        </is>
+      </c>
+      <c r="D1627" s="17" t="inlineStr">
+        <is>
+          <t>CHECK BANNER</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1628" s="17" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="C1628" s="17" t="inlineStr">
+        <is>
+          <t>Ask Banner</t>
+        </is>
+      </c>
+      <c r="D1628" s="17" t="inlineStr">
+        <is>
+          <t>Banner's auth tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1629" s="17" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C1629" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS Online / fax 602-256-6591</t>
+        </is>
+      </c>
+      <c r="D1629" s="17" t="inlineStr">
+        <is>
+          <t>AHCCCS Online</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" s="17" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B1630" s="17" t="inlineStr">
+        <is>
+          <t>A43</t>
+        </is>
+      </c>
+      <c r="C1630" s="17" t="inlineStr">
+        <is>
+          <t>- TPA groups (AHG, AmeriBen), BCBS SC, CHS, BlueCard home plans, Banner, delegated IPAs: call and record.</t>
+        </is>
+      </c>
+      <c r="D1630" s="17" t="inlineStr">
+        <is>
+          <t>- TPA groups (AHG, AmeriBen), BCBS SC, CHS, BlueCard home plans, Banner, delegated IPAs: check each one's auth tool and record the result.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>